<commit_message>
generalized informataion to ranges in TEstsceanrios, updated RAG information and building, clarified and consoldiated redundant functions, standardized timing and changed the start time, and removed some backups
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_shower.xlsx
+++ b/Ground Truth/ground_truth_shower.xlsx
@@ -626,13 +626,13 @@
         <v>10</v>
       </c>
       <c r="M3" t="n">
-        <v>5.63</v>
+        <v>4.76</v>
       </c>
       <c r="N3" t="n">
         <v>3.48</v>
       </c>
       <c r="O3" t="n">
-        <v>7.977</v>
+        <v>7.803</v>
       </c>
       <c r="P3" t="n">
         <v>2</v>
@@ -693,13 +693,13 @@
         <v>9.33</v>
       </c>
       <c r="M4" t="n">
-        <v>8.56</v>
+        <v>7.11</v>
       </c>
       <c r="N4" t="n">
         <v>7.6</v>
       </c>
       <c r="O4" t="n">
-        <v>8.6435</v>
+        <v>8.3535</v>
       </c>
       <c r="P4" t="n">
         <v>1</v>
@@ -961,16 +961,16 @@
         <v>10</v>
       </c>
       <c r="M8" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N8" t="n">
         <v>3.48</v>
       </c>
       <c r="O8" t="n">
-        <v>8.337</v>
+        <v>8.190999999999999</v>
       </c>
       <c r="P8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q8" t="n">
         <v>1.19415490086141</v>
@@ -1028,13 +1028,13 @@
         <v>9.33</v>
       </c>
       <c r="M9" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N9" t="n">
         <v>7.6</v>
       </c>
       <c r="O9" t="n">
-        <v>8.923499999999999</v>
+        <v>8.669499999999999</v>
       </c>
       <c r="P9" t="n">
         <v>1</v>
@@ -1095,16 +1095,16 @@
         <v>8.44</v>
       </c>
       <c r="M10" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N10" t="n">
         <v>9.25</v>
       </c>
       <c r="O10" t="n">
-        <v>8.307499999999999</v>
+        <v>8.3675</v>
       </c>
       <c r="P10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q10" t="n">
         <v>2.865971762067384</v>
@@ -1564,13 +1564,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M17" t="n">
-        <v>8.42</v>
+        <v>7.4</v>
       </c>
       <c r="N17" t="n">
         <v>5.01</v>
       </c>
       <c r="O17" t="n">
-        <v>7.872</v>
+        <v>7.668</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
@@ -1631,13 +1631,13 @@
         <v>7.78</v>
       </c>
       <c r="M18" t="n">
-        <v>9.369999999999999</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="N18" t="n">
         <v>5.19</v>
       </c>
       <c r="O18" t="n">
-        <v>7.196499999999999</v>
+        <v>7.0945</v>
       </c>
       <c r="P18" t="n">
         <v>2</v>
@@ -1698,13 +1698,13 @@
         <v>6.67</v>
       </c>
       <c r="M19" t="n">
-        <v>7.62</v>
+        <v>7.97</v>
       </c>
       <c r="N19" t="n">
         <v>6.69</v>
       </c>
       <c r="O19" t="n">
-        <v>6.178999999999999</v>
+        <v>6.249</v>
       </c>
       <c r="P19" t="n">
         <v>3</v>
@@ -1765,13 +1765,13 @@
         <v>10</v>
       </c>
       <c r="M20" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N20" t="n">
         <v>3.48</v>
       </c>
       <c r="O20" t="n">
-        <v>8.337</v>
+        <v>8.190999999999999</v>
       </c>
       <c r="P20" t="n">
         <v>3</v>
@@ -1832,16 +1832,16 @@
         <v>9.56</v>
       </c>
       <c r="M21" t="n">
-        <v>9.32</v>
+        <v>8.07</v>
       </c>
       <c r="N21" t="n">
         <v>6.37</v>
       </c>
       <c r="O21" t="n">
-        <v>8.7935</v>
+        <v>8.5435</v>
       </c>
       <c r="P21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q21" t="n">
         <v>1.671816861205974</v>
@@ -1899,16 +1899,16 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M22" t="n">
-        <v>9.59</v>
+        <v>9.85</v>
       </c>
       <c r="N22" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O22" t="n">
-        <v>8.622</v>
+        <v>8.673999999999999</v>
       </c>
       <c r="P22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q22" t="n">
         <v>2.38830980172282</v>
@@ -2033,13 +2033,13 @@
         <v>9.779999999999999</v>
       </c>
       <c r="M24" t="n">
-        <v>8.42</v>
+        <v>7.4</v>
       </c>
       <c r="N24" t="n">
         <v>5.01</v>
       </c>
       <c r="O24" t="n">
-        <v>8.5855</v>
+        <v>8.381499999999999</v>
       </c>
       <c r="P24" t="n">
         <v>1</v>
@@ -2100,13 +2100,13 @@
         <v>9.109999999999999</v>
       </c>
       <c r="M25" t="n">
-        <v>9.369999999999999</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="N25" t="n">
         <v>5.19</v>
       </c>
       <c r="O25" t="n">
-        <v>8.267999999999999</v>
+        <v>8.165999999999999</v>
       </c>
       <c r="P25" t="n">
         <v>2</v>
@@ -2368,13 +2368,13 @@
         <v>6.96</v>
       </c>
       <c r="M29" t="n">
-        <v>9.220000000000001</v>
+        <v>7.85</v>
       </c>
       <c r="N29" t="n">
         <v>4.64</v>
       </c>
       <c r="O29" t="n">
-        <v>6.428</v>
+        <v>6.154</v>
       </c>
       <c r="P29" t="n">
         <v>1</v>
@@ -2435,13 +2435,13 @@
         <v>4.89</v>
       </c>
       <c r="M30" t="n">
-        <v>6.77</v>
+        <v>7.15</v>
       </c>
       <c r="N30" t="n">
         <v>6.69</v>
       </c>
       <c r="O30" t="n">
-        <v>4.579</v>
+        <v>4.655</v>
       </c>
       <c r="P30" t="n">
         <v>2</v>
@@ -2770,13 +2770,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M35" t="n">
-        <v>8.42</v>
+        <v>7.4</v>
       </c>
       <c r="N35" t="n">
         <v>5.01</v>
       </c>
       <c r="O35" t="n">
-        <v>7.872</v>
+        <v>7.668</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
@@ -2837,13 +2837,13 @@
         <v>7.41</v>
       </c>
       <c r="M36" t="n">
-        <v>8.82</v>
+        <v>9.09</v>
       </c>
       <c r="N36" t="n">
         <v>5.71</v>
       </c>
       <c r="O36" t="n">
-        <v>6.866999999999999</v>
+        <v>6.920999999999998</v>
       </c>
       <c r="P36" t="n">
         <v>2</v>
@@ -3172,13 +3172,13 @@
         <v>8</v>
       </c>
       <c r="M41" t="n">
-        <v>8.42</v>
+        <v>7.4</v>
       </c>
       <c r="N41" t="n">
         <v>1.51</v>
       </c>
       <c r="O41" t="n">
-        <v>6.6335</v>
+        <v>6.4295</v>
       </c>
       <c r="P41" t="n">
         <v>1</v>
@@ -3239,13 +3239,13 @@
         <v>5.93</v>
       </c>
       <c r="M42" t="n">
-        <v>8.82</v>
+        <v>9.09</v>
       </c>
       <c r="N42" t="n">
         <v>5.71</v>
       </c>
       <c r="O42" t="n">
-        <v>5.677</v>
+        <v>5.730999999999999</v>
       </c>
       <c r="P42" t="n">
         <v>2</v>
@@ -3574,13 +3574,13 @@
         <v>4</v>
       </c>
       <c r="M47" t="n">
-        <v>6.77</v>
+        <v>7.15</v>
       </c>
       <c r="N47" t="n">
         <v>6.69</v>
       </c>
       <c r="O47" t="n">
-        <v>3.8625</v>
+        <v>3.9385</v>
       </c>
       <c r="P47" t="n">
         <v>1</v>
@@ -4253,7 +4253,7 @@
         <v>7.332999999999999</v>
       </c>
       <c r="P57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q57" t="n">
         <v>0.955323920689128</v>
@@ -4311,16 +4311,16 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M58" t="n">
-        <v>5.63</v>
+        <v>4.76</v>
       </c>
       <c r="N58" t="n">
         <v>1.51</v>
       </c>
       <c r="O58" t="n">
-        <v>7.383999999999999</v>
+        <v>7.209999999999999</v>
       </c>
       <c r="P58" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q58" t="n">
         <v>1.59220653448188</v>
@@ -4579,13 +4579,13 @@
         <v>7.56</v>
       </c>
       <c r="M62" t="n">
-        <v>9.9</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="N62" t="n">
         <v>4.64</v>
       </c>
       <c r="O62" t="n">
-        <v>7.041</v>
+        <v>6.785</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
@@ -4646,13 +4646,13 @@
         <v>5.78</v>
       </c>
       <c r="M63" t="n">
-        <v>7.62</v>
+        <v>7.97</v>
       </c>
       <c r="N63" t="n">
         <v>6.69</v>
       </c>
       <c r="O63" t="n">
-        <v>5.462499999999999</v>
+        <v>5.5325</v>
       </c>
       <c r="P63" t="n">
         <v>2</v>
@@ -4981,13 +4981,13 @@
         <v>8.52</v>
       </c>
       <c r="M68" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N68" t="n">
         <v>1.51</v>
       </c>
       <c r="O68" t="n">
-        <v>6.851499999999999</v>
+        <v>6.705499999999999</v>
       </c>
       <c r="P68" t="n">
         <v>1</v>
@@ -5048,13 +5048,13 @@
         <v>6.96</v>
       </c>
       <c r="M69" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N69" t="n">
         <v>4.64</v>
       </c>
       <c r="O69" t="n">
-        <v>6.576</v>
+        <v>6.321999999999999</v>
       </c>
       <c r="P69" t="n">
         <v>2</v>
@@ -5115,13 +5115,13 @@
         <v>4.89</v>
       </c>
       <c r="M70" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N70" t="n">
         <v>6.69</v>
       </c>
       <c r="O70" t="n">
-        <v>5.067</v>
+        <v>5.127</v>
       </c>
       <c r="P70" t="n">
         <v>3</v>
@@ -5182,13 +5182,13 @@
         <v>9.039999999999999</v>
       </c>
       <c r="M71" t="n">
-        <v>6.34</v>
+        <v>6.26</v>
       </c>
       <c r="N71" t="n">
         <v>2.86</v>
       </c>
       <c r="O71" t="n">
-        <v>7.531</v>
+        <v>7.515</v>
       </c>
       <c r="P71" t="n">
         <v>1</v>
@@ -5249,13 +5249,13 @@
         <v>7.48</v>
       </c>
       <c r="M72" t="n">
-        <v>9.32</v>
+        <v>9.08</v>
       </c>
       <c r="N72" t="n">
         <v>3.07</v>
       </c>
       <c r="O72" t="n">
-        <v>7.1145</v>
+        <v>7.0665</v>
       </c>
       <c r="P72" t="n">
         <v>2</v>
@@ -5316,13 +5316,13 @@
         <v>5.93</v>
       </c>
       <c r="M73" t="n">
-        <v>9.59</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="N73" t="n">
         <v>5.71</v>
       </c>
       <c r="O73" t="n">
-        <v>6.524</v>
+        <v>6.534</v>
       </c>
       <c r="P73" t="n">
         <v>3</v>
@@ -5383,13 +5383,13 @@
         <v>8.74</v>
       </c>
       <c r="M74" t="n">
-        <v>6.34</v>
+        <v>6.07</v>
       </c>
       <c r="N74" t="n">
         <v>2.86</v>
       </c>
       <c r="O74" t="n">
-        <v>7.204</v>
+        <v>7.15</v>
       </c>
       <c r="P74" t="n">
         <v>1</v>
@@ -5450,13 +5450,13 @@
         <v>6.96</v>
       </c>
       <c r="M75" t="n">
-        <v>9.32</v>
+        <v>8.49</v>
       </c>
       <c r="N75" t="n">
         <v>3.07</v>
       </c>
       <c r="O75" t="n">
-        <v>6.5485</v>
+        <v>6.3825</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
@@ -5517,13 +5517,13 @@
         <v>5.19</v>
       </c>
       <c r="M76" t="n">
-        <v>8.82</v>
+        <v>9.07</v>
       </c>
       <c r="N76" t="n">
         <v>5.71</v>
       </c>
       <c r="O76" t="n">
-        <v>5.562</v>
+        <v>5.611999999999999</v>
       </c>
       <c r="P76" t="n">
         <v>3</v>
@@ -5651,13 +5651,13 @@
         <v>8.74</v>
       </c>
       <c r="M78" t="n">
-        <v>9.9</v>
+        <v>9.24</v>
       </c>
       <c r="N78" t="n">
         <v>4.64</v>
       </c>
       <c r="O78" t="n">
-        <v>8.210000000000001</v>
+        <v>8.077999999999999</v>
       </c>
       <c r="P78" t="n">
         <v>1</v>
@@ -5785,13 +5785,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M80" t="n">
-        <v>6.34</v>
+        <v>6.19</v>
       </c>
       <c r="N80" t="n">
         <v>2.86</v>
       </c>
       <c r="O80" t="n">
-        <v>7.899500000000001</v>
+        <v>7.869500000000001</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -5852,13 +5852,13 @@
         <v>7.41</v>
       </c>
       <c r="M81" t="n">
-        <v>9.59</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="N81" t="n">
         <v>5.71</v>
       </c>
       <c r="O81" t="n">
-        <v>7.449999999999999</v>
+        <v>7.471999999999999</v>
       </c>
       <c r="P81" t="n">
         <v>2</v>
@@ -5986,13 +5986,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M83" t="n">
-        <v>7.43</v>
+        <v>6.85</v>
       </c>
       <c r="N83" t="n">
         <v>3.48</v>
       </c>
       <c r="O83" t="n">
-        <v>8.1325</v>
+        <v>8.016500000000001</v>
       </c>
       <c r="P83" t="n">
         <v>1</v>
@@ -6053,13 +6053,13 @@
         <v>7.56</v>
       </c>
       <c r="M84" t="n">
-        <v>7.62</v>
+        <v>7.84</v>
       </c>
       <c r="N84" t="n">
         <v>6.69</v>
       </c>
       <c r="O84" t="n">
-        <v>7.1175</v>
+        <v>7.161499999999999</v>
       </c>
       <c r="P84" t="n">
         <v>2</v>
@@ -6254,13 +6254,13 @@
         <v>8.52</v>
       </c>
       <c r="M87" t="n">
-        <v>9.32</v>
+        <v>8.07</v>
       </c>
       <c r="N87" t="n">
         <v>6.37</v>
       </c>
       <c r="O87" t="n">
-        <v>8.0305</v>
+        <v>7.780499999999999</v>
       </c>
       <c r="P87" t="n">
         <v>1</v>
@@ -6321,13 +6321,13 @@
         <v>5.93</v>
       </c>
       <c r="M88" t="n">
-        <v>8.81</v>
+        <v>8.92</v>
       </c>
       <c r="N88" t="n">
         <v>5.71</v>
       </c>
       <c r="O88" t="n">
-        <v>5.819</v>
+        <v>5.840999999999999</v>
       </c>
       <c r="P88" t="n">
         <v>3</v>
@@ -6388,13 +6388,13 @@
         <v>9.33</v>
       </c>
       <c r="M89" t="n">
-        <v>8.42</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="N89" t="n">
         <v>5.01</v>
       </c>
       <c r="O89" t="n">
-        <v>8.478999999999999</v>
+        <v>8.452999999999999</v>
       </c>
       <c r="P89" t="n">
         <v>1</v>
@@ -6455,13 +6455,13 @@
         <v>8.15</v>
       </c>
       <c r="M90" t="n">
-        <v>9.59</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="N90" t="n">
         <v>5.71</v>
       </c>
       <c r="O90" t="n">
-        <v>8.032999999999999</v>
+        <v>8.039</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
@@ -6589,13 +6589,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M92" t="n">
-        <v>5.63</v>
+        <v>4.98</v>
       </c>
       <c r="N92" t="n">
         <v>3.48</v>
       </c>
       <c r="O92" t="n">
-        <v>7.7845</v>
+        <v>7.654500000000001</v>
       </c>
       <c r="P92" t="n">
         <v>2</v>
@@ -6656,13 +6656,13 @@
         <v>8.74</v>
       </c>
       <c r="M93" t="n">
-        <v>8.56</v>
+        <v>7.55</v>
       </c>
       <c r="N93" t="n">
         <v>7.6</v>
       </c>
       <c r="O93" t="n">
-        <v>8.335000000000001</v>
+        <v>8.132999999999999</v>
       </c>
       <c r="P93" t="n">
         <v>1</v>
@@ -6723,13 +6723,13 @@
         <v>7.56</v>
       </c>
       <c r="M94" t="n">
-        <v>7.7</v>
+        <v>7.9</v>
       </c>
       <c r="N94" t="n">
         <v>6.69</v>
       </c>
       <c r="O94" t="n">
-        <v>7.1605</v>
+        <v>7.2005</v>
       </c>
       <c r="P94" t="n">
         <v>3</v>
@@ -6790,13 +6790,13 @@
         <v>9.26</v>
       </c>
       <c r="M95" t="n">
-        <v>5.63</v>
+        <v>4.84</v>
       </c>
       <c r="N95" t="n">
         <v>3.48</v>
       </c>
       <c r="O95" t="n">
-        <v>7.466</v>
+        <v>7.308</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
@@ -6857,13 +6857,13 @@
         <v>8.15</v>
       </c>
       <c r="M96" t="n">
-        <v>8.56</v>
+        <v>7.27</v>
       </c>
       <c r="N96" t="n">
         <v>4.64</v>
       </c>
       <c r="O96" t="n">
-        <v>7.384499999999999</v>
+        <v>7.126499999999999</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
@@ -6924,13 +6924,13 @@
         <v>6.67</v>
       </c>
       <c r="M97" t="n">
-        <v>7.7</v>
+        <v>7.99</v>
       </c>
       <c r="N97" t="n">
         <v>6.69</v>
       </c>
       <c r="O97" t="n">
-        <v>6.399</v>
+        <v>6.457</v>
       </c>
       <c r="P97" t="n">
         <v>3</v>
@@ -6991,13 +6991,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M98" t="n">
-        <v>7.43</v>
+        <v>7.04</v>
       </c>
       <c r="N98" t="n">
         <v>3.48</v>
       </c>
       <c r="O98" t="n">
-        <v>8.186499999999999</v>
+        <v>8.108499999999999</v>
       </c>
       <c r="P98" t="n">
         <v>2</v>
@@ -7058,13 +7058,13 @@
         <v>8.74</v>
       </c>
       <c r="M99" t="n">
-        <v>9.960000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="N99" t="n">
         <v>7.6</v>
       </c>
       <c r="O99" t="n">
-        <v>8.680999999999999</v>
+        <v>8.567</v>
       </c>
       <c r="P99" t="n">
         <v>1</v>
@@ -7125,13 +7125,13 @@
         <v>7.56</v>
       </c>
       <c r="M100" t="n">
-        <v>9.210000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="N100" t="n">
         <v>6.69</v>
       </c>
       <c r="O100" t="n">
-        <v>7.5615</v>
+        <v>7.581499999999999</v>
       </c>
       <c r="P100" t="n">
         <v>3</v>
@@ -7192,13 +7192,13 @@
         <v>9.26</v>
       </c>
       <c r="M101" t="n">
-        <v>7.43</v>
+        <v>6.94</v>
       </c>
       <c r="N101" t="n">
         <v>3.48</v>
       </c>
       <c r="O101" t="n">
-        <v>7.892</v>
+        <v>7.794</v>
       </c>
       <c r="P101" t="n">
         <v>2</v>
@@ -7259,13 +7259,13 @@
         <v>8.15</v>
       </c>
       <c r="M102" t="n">
-        <v>9.960000000000001</v>
+        <v>9.19</v>
       </c>
       <c r="N102" t="n">
         <v>7.6</v>
       </c>
       <c r="O102" t="n">
-        <v>8.2135</v>
+        <v>8.0595</v>
       </c>
       <c r="P102" t="n">
         <v>1</v>
@@ -7326,13 +7326,13 @@
         <v>6.67</v>
       </c>
       <c r="M103" t="n">
-        <v>9.210000000000001</v>
+        <v>9.35</v>
       </c>
       <c r="N103" t="n">
         <v>6.69</v>
       </c>
       <c r="O103" t="n">
-        <v>6.857</v>
+        <v>6.885</v>
       </c>
       <c r="P103" t="n">
         <v>3</v>
@@ -7393,13 +7393,13 @@
         <v>9.26</v>
       </c>
       <c r="M104" t="n">
-        <v>6.57</v>
+        <v>5.9</v>
       </c>
       <c r="N104" t="n">
         <v>3.48</v>
       </c>
       <c r="O104" t="n">
-        <v>7.675</v>
+        <v>7.541</v>
       </c>
       <c r="P104" t="n">
         <v>1</v>
@@ -7460,13 +7460,13 @@
         <v>8.15</v>
       </c>
       <c r="M105" t="n">
-        <v>9.220000000000001</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="N105" t="n">
         <v>4.64</v>
       </c>
       <c r="O105" t="n">
-        <v>7.5495</v>
+        <v>7.3275</v>
       </c>
       <c r="P105" t="n">
         <v>2</v>
@@ -7527,13 +7527,13 @@
         <v>6.67</v>
       </c>
       <c r="M106" t="n">
-        <v>6.77</v>
+        <v>7.04</v>
       </c>
       <c r="N106" t="n">
         <v>6.69</v>
       </c>
       <c r="O106" t="n">
-        <v>6.258</v>
+        <v>6.311999999999999</v>
       </c>
       <c r="P106" t="n">
         <v>3</v>
@@ -7594,13 +7594,13 @@
         <v>8.15</v>
       </c>
       <c r="M107" t="n">
-        <v>9.9</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N107" t="n">
         <v>4.64</v>
       </c>
       <c r="O107" t="n">
-        <v>7.7575</v>
+        <v>7.6015</v>
       </c>
       <c r="P107" t="n">
         <v>1</v>
@@ -7661,13 +7661,13 @@
         <v>7.41</v>
       </c>
       <c r="M108" t="n">
-        <v>8.82</v>
+        <v>9.07</v>
       </c>
       <c r="N108" t="n">
         <v>5.71</v>
       </c>
       <c r="O108" t="n">
-        <v>7.167</v>
+        <v>7.217</v>
       </c>
       <c r="P108" t="n">
         <v>2</v>
@@ -7728,13 +7728,13 @@
         <v>6.67</v>
       </c>
       <c r="M109" t="n">
-        <v>7.62</v>
+        <v>7.79</v>
       </c>
       <c r="N109" t="n">
         <v>6.69</v>
       </c>
       <c r="O109" t="n">
-        <v>6.539</v>
+        <v>6.573</v>
       </c>
       <c r="P109" t="n">
         <v>3</v>
@@ -7795,13 +7795,13 @@
         <v>7.56</v>
       </c>
       <c r="M110" t="n">
-        <v>9.9</v>
+        <v>8.93</v>
       </c>
       <c r="N110" t="n">
         <v>4.64</v>
       </c>
       <c r="O110" t="n">
-        <v>7.266</v>
+        <v>7.071999999999999</v>
       </c>
       <c r="P110" t="n">
         <v>1</v>
@@ -7862,13 +7862,13 @@
         <v>6.67</v>
       </c>
       <c r="M111" t="n">
-        <v>8.82</v>
+        <v>9.15</v>
       </c>
       <c r="N111" t="n">
         <v>5.71</v>
       </c>
       <c r="O111" t="n">
-        <v>6.553999999999999</v>
+        <v>6.619999999999999</v>
       </c>
       <c r="P111" t="n">
         <v>2</v>
@@ -7929,13 +7929,13 @@
         <v>5.78</v>
       </c>
       <c r="M112" t="n">
-        <v>7.62</v>
+        <v>7.84</v>
       </c>
       <c r="N112" t="n">
         <v>6.69</v>
       </c>
       <c r="O112" t="n">
-        <v>5.8015</v>
+        <v>5.8455</v>
       </c>
       <c r="P112" t="n">
         <v>3</v>
@@ -7996,13 +7996,13 @@
         <v>8.15</v>
       </c>
       <c r="M113" t="n">
-        <v>9.9</v>
+        <v>9.32</v>
       </c>
       <c r="N113" t="n">
         <v>4.64</v>
       </c>
       <c r="O113" t="n">
-        <v>7.8085</v>
+        <v>7.6925</v>
       </c>
       <c r="P113" t="n">
         <v>1</v>
@@ -8063,13 +8063,13 @@
         <v>7.41</v>
       </c>
       <c r="M114" t="n">
-        <v>8.82</v>
+        <v>9</v>
       </c>
       <c r="N114" t="n">
         <v>5.71</v>
       </c>
       <c r="O114" t="n">
-        <v>7.23</v>
+        <v>7.265999999999999</v>
       </c>
       <c r="P114" t="n">
         <v>2</v>
@@ -8130,13 +8130,13 @@
         <v>6.67</v>
       </c>
       <c r="M115" t="n">
-        <v>7.62</v>
+        <v>7.74</v>
       </c>
       <c r="N115" t="n">
         <v>6.69</v>
       </c>
       <c r="O115" t="n">
-        <v>6.616999999999999</v>
+        <v>6.640999999999999</v>
       </c>
       <c r="P115" t="n">
         <v>3</v>
@@ -8197,13 +8197,13 @@
         <v>8.74</v>
       </c>
       <c r="M116" t="n">
-        <v>9.9</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N116" t="n">
         <v>4.64</v>
       </c>
       <c r="O116" t="n">
-        <v>8.183</v>
+        <v>8.026999999999999</v>
       </c>
       <c r="P116" t="n">
         <v>1</v>
@@ -8264,13 +8264,13 @@
         <v>8.15</v>
       </c>
       <c r="M117" t="n">
-        <v>8.82</v>
+        <v>9.07</v>
       </c>
       <c r="N117" t="n">
         <v>5.71</v>
       </c>
       <c r="O117" t="n">
-        <v>7.702</v>
+        <v>7.752</v>
       </c>
       <c r="P117" t="n">
         <v>2</v>
@@ -8331,13 +8331,13 @@
         <v>7.56</v>
       </c>
       <c r="M118" t="n">
-        <v>7.62</v>
+        <v>7.79</v>
       </c>
       <c r="N118" t="n">
         <v>6.69</v>
       </c>
       <c r="O118" t="n">
-        <v>7.1805</v>
+        <v>7.2145</v>
       </c>
       <c r="P118" t="n">
         <v>3</v>
@@ -8398,13 +8398,13 @@
         <v>8.15</v>
       </c>
       <c r="M119" t="n">
-        <v>9.9</v>
+        <v>9.24</v>
       </c>
       <c r="N119" t="n">
         <v>4.64</v>
       </c>
       <c r="O119" t="n">
-        <v>7.7875</v>
+        <v>7.655499999999999</v>
       </c>
       <c r="P119" t="n">
         <v>1</v>
@@ -8465,13 +8465,13 @@
         <v>7.41</v>
       </c>
       <c r="M120" t="n">
-        <v>8.82</v>
+        <v>9.02</v>
       </c>
       <c r="N120" t="n">
         <v>5.71</v>
       </c>
       <c r="O120" t="n">
-        <v>7.206</v>
+        <v>7.246</v>
       </c>
       <c r="P120" t="n">
         <v>2</v>
@@ -8532,13 +8532,13 @@
         <v>6.67</v>
       </c>
       <c r="M121" t="n">
-        <v>7.62</v>
+        <v>7.76</v>
       </c>
       <c r="N121" t="n">
         <v>6.69</v>
       </c>
       <c r="O121" t="n">
-        <v>6.584</v>
+        <v>6.611999999999999</v>
       </c>
       <c r="P121" t="n">
         <v>3</v>
@@ -8599,13 +8599,13 @@
         <v>9.26</v>
       </c>
       <c r="M122" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N122" t="n">
         <v>3.48</v>
       </c>
       <c r="O122" t="n">
-        <v>7.742</v>
+        <v>7.596</v>
       </c>
       <c r="P122" t="n">
         <v>1</v>
@@ -8666,13 +8666,13 @@
         <v>8.15</v>
       </c>
       <c r="M123" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N123" t="n">
         <v>4.64</v>
       </c>
       <c r="O123" t="n">
-        <v>7.5295</v>
+        <v>7.275499999999999</v>
       </c>
       <c r="P123" t="n">
         <v>2</v>
@@ -8733,13 +8733,13 @@
         <v>6.67</v>
       </c>
       <c r="M124" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N124" t="n">
         <v>6.69</v>
       </c>
       <c r="O124" t="n">
-        <v>6.497</v>
+        <v>6.556999999999999</v>
       </c>
       <c r="P124" t="n">
         <v>3</v>
@@ -8800,13 +8800,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M125" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N125" t="n">
         <v>3.48</v>
       </c>
       <c r="O125" t="n">
-        <v>8.039499999999999</v>
+        <v>7.8935</v>
       </c>
       <c r="P125" t="n">
         <v>2</v>
@@ -8867,13 +8867,13 @@
         <v>8.74</v>
       </c>
       <c r="M126" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N126" t="n">
         <v>7.6</v>
       </c>
       <c r="O126" t="n">
-        <v>8.449999999999999</v>
+        <v>8.196</v>
       </c>
       <c r="P126" t="n">
         <v>1</v>
@@ -8934,13 +8934,13 @@
         <v>7.56</v>
       </c>
       <c r="M127" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N127" t="n">
         <v>6.69</v>
       </c>
       <c r="O127" t="n">
-        <v>7.210500000000001</v>
+        <v>7.2705</v>
       </c>
       <c r="P127" t="n">
         <v>3</v>
@@ -9001,13 +9001,13 @@
         <v>9.26</v>
       </c>
       <c r="M128" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N128" t="n">
         <v>3.48</v>
       </c>
       <c r="O128" t="n">
-        <v>7.742</v>
+        <v>7.596</v>
       </c>
       <c r="P128" t="n">
         <v>1</v>
@@ -9068,13 +9068,13 @@
         <v>8.15</v>
       </c>
       <c r="M129" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N129" t="n">
         <v>4.64</v>
       </c>
       <c r="O129" t="n">
-        <v>7.5295</v>
+        <v>7.275499999999999</v>
       </c>
       <c r="P129" t="n">
         <v>2</v>
@@ -9135,13 +9135,13 @@
         <v>6.67</v>
       </c>
       <c r="M130" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N130" t="n">
         <v>6.69</v>
       </c>
       <c r="O130" t="n">
-        <v>6.497</v>
+        <v>6.556999999999999</v>
       </c>
       <c r="P130" t="n">
         <v>3</v>
@@ -9604,13 +9604,13 @@
         <v>9.33</v>
       </c>
       <c r="M137" t="n">
-        <v>6.34</v>
+        <v>5.95</v>
       </c>
       <c r="N137" t="n">
         <v>2.86</v>
       </c>
       <c r="O137" t="n">
-        <v>7.5515</v>
+        <v>7.4735</v>
       </c>
       <c r="P137" t="n">
         <v>1</v>
@@ -9671,13 +9671,13 @@
         <v>8</v>
       </c>
       <c r="M138" t="n">
-        <v>9.32</v>
+        <v>8.1</v>
       </c>
       <c r="N138" t="n">
         <v>3.07</v>
       </c>
       <c r="O138" t="n">
-        <v>7.155499999999999</v>
+        <v>6.911499999999999</v>
       </c>
       <c r="P138" t="n">
         <v>2</v>
@@ -9738,13 +9738,13 @@
         <v>6.67</v>
       </c>
       <c r="M139" t="n">
-        <v>9.59</v>
+        <v>9.9</v>
       </c>
       <c r="N139" t="n">
         <v>5.71</v>
       </c>
       <c r="O139" t="n">
-        <v>6.582</v>
+        <v>6.644</v>
       </c>
       <c r="P139" t="n">
         <v>3</v>
@@ -9805,13 +9805,13 @@
         <v>8.74</v>
       </c>
       <c r="M140" t="n">
-        <v>6.34</v>
+        <v>5.94</v>
       </c>
       <c r="N140" t="n">
         <v>1.51</v>
       </c>
       <c r="O140" t="n">
-        <v>6.860499999999999</v>
+        <v>6.7805</v>
       </c>
       <c r="P140" t="n">
         <v>1</v>
@@ -9872,13 +9872,13 @@
         <v>6.96</v>
       </c>
       <c r="M141" t="n">
-        <v>9.32</v>
+        <v>8.07</v>
       </c>
       <c r="N141" t="n">
         <v>3.07</v>
       </c>
       <c r="O141" t="n">
-        <v>6.299499999999999</v>
+        <v>6.049499999999999</v>
       </c>
       <c r="P141" t="n">
         <v>2</v>
@@ -9939,13 +9939,13 @@
         <v>5.19</v>
       </c>
       <c r="M142" t="n">
-        <v>8.82</v>
+        <v>9.09</v>
       </c>
       <c r="N142" t="n">
         <v>5.71</v>
       </c>
       <c r="O142" t="n">
-        <v>5.205</v>
+        <v>5.258999999999999</v>
       </c>
       <c r="P142" t="n">
         <v>3</v>
@@ -10073,13 +10073,13 @@
         <v>9.33</v>
       </c>
       <c r="M144" t="n">
-        <v>8.42</v>
+        <v>7.74</v>
       </c>
       <c r="N144" t="n">
         <v>5.01</v>
       </c>
       <c r="O144" t="n">
-        <v>8.370999999999999</v>
+        <v>8.234999999999999</v>
       </c>
       <c r="P144" t="n">
         <v>1</v>
@@ -10140,13 +10140,13 @@
         <v>7.56</v>
       </c>
       <c r="M145" t="n">
-        <v>9.210000000000001</v>
+        <v>9.35</v>
       </c>
       <c r="N145" t="n">
         <v>6.69</v>
       </c>
       <c r="O145" t="n">
-        <v>7.498500000000001</v>
+        <v>7.5265</v>
       </c>
       <c r="P145" t="n">
         <v>2</v>
@@ -10207,13 +10207,13 @@
         <v>8.52</v>
       </c>
       <c r="M146" t="n">
-        <v>9.32</v>
+        <v>8.74</v>
       </c>
       <c r="N146" t="n">
         <v>6.37</v>
       </c>
       <c r="O146" t="n">
-        <v>8.231499999999999</v>
+        <v>8.115499999999999</v>
       </c>
       <c r="P146" t="n">
         <v>1</v>
@@ -10274,13 +10274,13 @@
         <v>5.93</v>
       </c>
       <c r="M147" t="n">
-        <v>8.81</v>
+        <v>8.84</v>
       </c>
       <c r="N147" t="n">
         <v>5.71</v>
       </c>
       <c r="O147" t="n">
-        <v>6.221</v>
+        <v>6.226999999999999</v>
       </c>
       <c r="P147" t="n">
         <v>2</v>
@@ -10408,13 +10408,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M149" t="n">
-        <v>5.63</v>
+        <v>4.94</v>
       </c>
       <c r="N149" t="n">
         <v>3.48</v>
       </c>
       <c r="O149" t="n">
-        <v>7.772500000000001</v>
+        <v>7.634500000000001</v>
       </c>
       <c r="P149" t="n">
         <v>2</v>
@@ -10475,13 +10475,13 @@
         <v>8.74</v>
       </c>
       <c r="M150" t="n">
-        <v>8.56</v>
+        <v>7.46</v>
       </c>
       <c r="N150" t="n">
         <v>4.64</v>
       </c>
       <c r="O150" t="n">
-        <v>7.875999999999999</v>
+        <v>7.656</v>
       </c>
       <c r="P150" t="n">
         <v>1</v>
@@ -10542,13 +10542,13 @@
         <v>7.56</v>
       </c>
       <c r="M151" t="n">
-        <v>7.7</v>
+        <v>7.92</v>
       </c>
       <c r="N151" t="n">
         <v>6.69</v>
       </c>
       <c r="O151" t="n">
-        <v>7.1335</v>
+        <v>7.177499999999999</v>
       </c>
       <c r="P151" t="n">
         <v>3</v>
@@ -10609,13 +10609,13 @@
         <v>9.26</v>
       </c>
       <c r="M152" t="n">
-        <v>6.57</v>
+        <v>6.1</v>
       </c>
       <c r="N152" t="n">
         <v>3.48</v>
       </c>
       <c r="O152" t="n">
-        <v>7.738</v>
+        <v>7.643999999999999</v>
       </c>
       <c r="P152" t="n">
         <v>2</v>
@@ -10676,13 +10676,13 @@
         <v>8.15</v>
       </c>
       <c r="M153" t="n">
-        <v>9.289999999999999</v>
+        <v>8.59</v>
       </c>
       <c r="N153" t="n">
         <v>7.6</v>
       </c>
       <c r="O153" t="n">
-        <v>8.109499999999999</v>
+        <v>7.969499999999999</v>
       </c>
       <c r="P153" t="n">
         <v>1</v>
@@ -10743,13 +10743,13 @@
         <v>6.67</v>
       </c>
       <c r="M154" t="n">
-        <v>8.48</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="N154" t="n">
         <v>6.69</v>
       </c>
       <c r="O154" t="n">
-        <v>6.755999999999999</v>
+        <v>6.781999999999999</v>
       </c>
       <c r="P154" t="n">
         <v>3</v>
@@ -10810,13 +10810,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M155" t="n">
-        <v>8.42</v>
+        <v>7.74</v>
       </c>
       <c r="N155" t="n">
         <v>1.51</v>
       </c>
       <c r="O155" t="n">
-        <v>7.527</v>
+        <v>7.391</v>
       </c>
       <c r="P155" t="n">
         <v>2</v>
@@ -10877,13 +10877,13 @@
         <v>8.15</v>
       </c>
       <c r="M156" t="n">
-        <v>9.9</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="N156" t="n">
         <v>4.64</v>
       </c>
       <c r="O156" t="n">
-        <v>7.7575</v>
+        <v>7.6015</v>
       </c>
       <c r="P156" t="n">
         <v>1</v>
@@ -10944,13 +10944,13 @@
         <v>7.41</v>
       </c>
       <c r="M157" t="n">
-        <v>8.82</v>
+        <v>9.07</v>
       </c>
       <c r="N157" t="n">
         <v>5.71</v>
       </c>
       <c r="O157" t="n">
-        <v>7.167</v>
+        <v>7.217</v>
       </c>
       <c r="P157" t="n">
         <v>3</v>
@@ -11011,13 +11011,13 @@
         <v>8.15</v>
       </c>
       <c r="M158" t="n">
-        <v>9.9</v>
+        <v>9.24</v>
       </c>
       <c r="N158" t="n">
         <v>4.64</v>
       </c>
       <c r="O158" t="n">
-        <v>7.7875</v>
+        <v>7.655499999999999</v>
       </c>
       <c r="P158" t="n">
         <v>1</v>
@@ -11078,13 +11078,13 @@
         <v>7.41</v>
       </c>
       <c r="M159" t="n">
-        <v>8.82</v>
+        <v>9.02</v>
       </c>
       <c r="N159" t="n">
         <v>5.71</v>
       </c>
       <c r="O159" t="n">
-        <v>7.206</v>
+        <v>7.246</v>
       </c>
       <c r="P159" t="n">
         <v>2</v>
@@ -11145,13 +11145,13 @@
         <v>6.67</v>
       </c>
       <c r="M160" t="n">
-        <v>7.62</v>
+        <v>7.76</v>
       </c>
       <c r="N160" t="n">
         <v>6.69</v>
       </c>
       <c r="O160" t="n">
-        <v>6.584</v>
+        <v>6.611999999999999</v>
       </c>
       <c r="P160" t="n">
         <v>3</v>
@@ -11212,13 +11212,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M161" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N161" t="n">
         <v>3.48</v>
       </c>
       <c r="O161" t="n">
-        <v>8.039499999999999</v>
+        <v>7.8935</v>
       </c>
       <c r="P161" t="n">
         <v>2</v>
@@ -11279,13 +11279,13 @@
         <v>8.74</v>
       </c>
       <c r="M162" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N162" t="n">
         <v>7.6</v>
       </c>
       <c r="O162" t="n">
-        <v>8.449999999999999</v>
+        <v>8.196</v>
       </c>
       <c r="P162" t="n">
         <v>1</v>
@@ -11346,13 +11346,13 @@
         <v>7.56</v>
       </c>
       <c r="M163" t="n">
-        <v>9.210000000000001</v>
+        <v>9.51</v>
       </c>
       <c r="N163" t="n">
         <v>6.69</v>
       </c>
       <c r="O163" t="n">
-        <v>7.210500000000001</v>
+        <v>7.2705</v>
       </c>
       <c r="P163" t="n">
         <v>3</v>
@@ -11681,13 +11681,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M168" t="n">
-        <v>7.43</v>
+        <v>7.15</v>
       </c>
       <c r="N168" t="n">
         <v>3.48</v>
       </c>
       <c r="O168" t="n">
-        <v>8.2105</v>
+        <v>8.154500000000001</v>
       </c>
       <c r="P168" t="n">
         <v>2</v>
@@ -11748,13 +11748,13 @@
         <v>8.74</v>
       </c>
       <c r="M169" t="n">
-        <v>9.960000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="N169" t="n">
         <v>7.6</v>
       </c>
       <c r="O169" t="n">
-        <v>8.722999999999999</v>
+        <v>8.654999999999999</v>
       </c>
       <c r="P169" t="n">
         <v>1</v>
@@ -12083,13 +12083,13 @@
         <v>9.26</v>
       </c>
       <c r="M174" t="n">
-        <v>7.43</v>
+        <v>7.34</v>
       </c>
       <c r="N174" t="n">
         <v>3.48</v>
       </c>
       <c r="O174" t="n">
-        <v>8.002999999999998</v>
+        <v>7.984999999999999</v>
       </c>
       <c r="P174" t="n">
         <v>1</v>
@@ -12150,13 +12150,13 @@
         <v>8.15</v>
       </c>
       <c r="M175" t="n">
-        <v>9.960000000000001</v>
+        <v>9.99</v>
       </c>
       <c r="N175" t="n">
         <v>4.64</v>
       </c>
       <c r="O175" t="n">
-        <v>7.946499999999999</v>
+        <v>7.9525</v>
       </c>
       <c r="P175" t="n">
         <v>2</v>
@@ -12284,13 +12284,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M177" t="n">
-        <v>7.43</v>
+        <v>7</v>
       </c>
       <c r="N177" t="n">
         <v>3.48</v>
       </c>
       <c r="O177" t="n">
-        <v>8.1745</v>
+        <v>8.0885</v>
       </c>
       <c r="P177" t="n">
         <v>2</v>
@@ -12351,13 +12351,13 @@
         <v>8.74</v>
       </c>
       <c r="M178" t="n">
-        <v>9.960000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="N178" t="n">
         <v>7.6</v>
       </c>
       <c r="O178" t="n">
-        <v>8.666</v>
+        <v>8.536</v>
       </c>
       <c r="P178" t="n">
         <v>1</v>
@@ -12418,13 +12418,13 @@
         <v>10</v>
       </c>
       <c r="M179" t="n">
-        <v>4.33</v>
+        <v>3.85</v>
       </c>
       <c r="N179" t="n">
         <v>2.86</v>
       </c>
       <c r="O179" t="n">
-        <v>7.734999999999999</v>
+        <v>7.638999999999999</v>
       </c>
       <c r="P179" t="n">
         <v>3</v>
@@ -12485,13 +12485,13 @@
         <v>9.779999999999999</v>
       </c>
       <c r="M180" t="n">
-        <v>6.79</v>
+        <v>5.6</v>
       </c>
       <c r="N180" t="n">
         <v>5.01</v>
       </c>
       <c r="O180" t="n">
-        <v>8.2745</v>
+        <v>8.036499999999998</v>
       </c>
       <c r="P180" t="n">
         <v>2</v>
@@ -12552,13 +12552,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M181" t="n">
-        <v>8.140000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="N181" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O181" t="n">
-        <v>8.356</v>
+        <v>8.414</v>
       </c>
       <c r="P181" t="n">
         <v>1</v>
@@ -12619,13 +12619,13 @@
         <v>9.93</v>
       </c>
       <c r="M182" t="n">
-        <v>6.34</v>
+        <v>6</v>
       </c>
       <c r="N182" t="n">
         <v>2.86</v>
       </c>
       <c r="O182" t="n">
-        <v>8.0345</v>
+        <v>7.9665</v>
       </c>
       <c r="P182" t="n">
         <v>3</v>
@@ -12686,16 +12686,16 @@
         <v>9.33</v>
       </c>
       <c r="M183" t="n">
-        <v>8.42</v>
+        <v>7.56</v>
       </c>
       <c r="N183" t="n">
         <v>5.01</v>
       </c>
       <c r="O183" t="n">
-        <v>8.328999999999999</v>
+        <v>8.157</v>
       </c>
       <c r="P183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q183" t="n">
         <v>1.673668264153046</v>
@@ -12753,16 +12753,16 @@
         <v>8.15</v>
       </c>
       <c r="M184" t="n">
-        <v>9.59</v>
+        <v>9.94</v>
       </c>
       <c r="N184" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O184" t="n">
-        <v>8.195</v>
+        <v>8.265000000000001</v>
       </c>
       <c r="P184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q184" t="n">
         <v>2.789447106921743</v>
@@ -12829,7 +12829,7 @@
         <v>7.802</v>
       </c>
       <c r="P185" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q185" t="n">
         <v>0.916444458800617</v>
@@ -12887,13 +12887,13 @@
         <v>9.26</v>
       </c>
       <c r="M186" t="n">
-        <v>7.43</v>
+        <v>7.08</v>
       </c>
       <c r="N186" t="n">
         <v>3.48</v>
       </c>
       <c r="O186" t="n">
-        <v>7.937</v>
+        <v>7.867000000000001</v>
       </c>
       <c r="P186" t="n">
         <v>1</v>
@@ -12954,16 +12954,16 @@
         <v>8.15</v>
       </c>
       <c r="M187" t="n">
-        <v>9.960000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="N187" t="n">
         <v>4.64</v>
       </c>
       <c r="O187" t="n">
-        <v>7.841499999999999</v>
+        <v>7.745499999999999</v>
       </c>
       <c r="P187" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q187" t="n">
         <v>2.443851890134979</v>
@@ -13088,13 +13088,13 @@
         <v>9.33</v>
       </c>
       <c r="M189" t="n">
-        <v>6.34</v>
+        <v>6.26</v>
       </c>
       <c r="N189" t="n">
         <v>2.86</v>
       </c>
       <c r="O189" t="n">
-        <v>7.7255</v>
+        <v>7.7095</v>
       </c>
       <c r="P189" t="n">
         <v>1</v>
@@ -13155,13 +13155,13 @@
         <v>8.44</v>
       </c>
       <c r="M190" t="n">
-        <v>8.42</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="N190" t="n">
         <v>1.51</v>
       </c>
       <c r="O190" t="n">
-        <v>7.345499999999999</v>
+        <v>7.305499999999999</v>
       </c>
       <c r="P190" t="n">
         <v>3</v>
@@ -13289,13 +13289,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M192" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N192" t="n">
         <v>3.48</v>
       </c>
       <c r="O192" t="n">
-        <v>8.039499999999999</v>
+        <v>7.8935</v>
       </c>
       <c r="P192" t="n">
         <v>2</v>
@@ -13356,13 +13356,13 @@
         <v>8.74</v>
       </c>
       <c r="M193" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N193" t="n">
         <v>7.6</v>
       </c>
       <c r="O193" t="n">
-        <v>8.449999999999999</v>
+        <v>8.196</v>
       </c>
       <c r="P193" t="n">
         <v>1</v>
@@ -13432,7 +13432,7 @@
         <v>7.802</v>
       </c>
       <c r="P194" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q194" t="n">
         <v>0.916444458800617</v>
@@ -13490,13 +13490,13 @@
         <v>9.26</v>
       </c>
       <c r="M195" t="n">
-        <v>7.43</v>
+        <v>7.08</v>
       </c>
       <c r="N195" t="n">
         <v>3.48</v>
       </c>
       <c r="O195" t="n">
-        <v>7.937</v>
+        <v>7.867000000000001</v>
       </c>
       <c r="P195" t="n">
         <v>1</v>
@@ -13557,16 +13557,16 @@
         <v>8.15</v>
       </c>
       <c r="M196" t="n">
-        <v>9.960000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="N196" t="n">
         <v>4.64</v>
       </c>
       <c r="O196" t="n">
-        <v>7.841499999999999</v>
+        <v>7.745499999999999</v>
       </c>
       <c r="P196" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q196" t="n">
         <v>2.443851890134979</v>
@@ -13892,13 +13892,13 @@
         <v>9.26</v>
       </c>
       <c r="M201" t="n">
-        <v>7.43</v>
+        <v>6.94</v>
       </c>
       <c r="N201" t="n">
         <v>3.48</v>
       </c>
       <c r="O201" t="n">
-        <v>7.892</v>
+        <v>7.794</v>
       </c>
       <c r="P201" t="n">
         <v>1</v>
@@ -13959,13 +13959,13 @@
         <v>8.52</v>
       </c>
       <c r="M202" t="n">
-        <v>9.32</v>
+        <v>8.49</v>
       </c>
       <c r="N202" t="n">
         <v>3.07</v>
       </c>
       <c r="O202" t="n">
-        <v>7.6735</v>
+        <v>7.5075</v>
       </c>
       <c r="P202" t="n">
         <v>3</v>
@@ -14093,13 +14093,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M204" t="n">
-        <v>7.43</v>
+        <v>7.08</v>
       </c>
       <c r="N204" t="n">
         <v>3.48</v>
       </c>
       <c r="O204" t="n">
-        <v>8.195499999999999</v>
+        <v>8.125500000000001</v>
       </c>
       <c r="P204" t="n">
         <v>2</v>
@@ -14160,13 +14160,13 @@
         <v>8.74</v>
       </c>
       <c r="M205" t="n">
-        <v>9.960000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="N205" t="n">
         <v>7.6</v>
       </c>
       <c r="O205" t="n">
-        <v>8.699</v>
+        <v>8.603</v>
       </c>
       <c r="P205" t="n">
         <v>1</v>
@@ -14236,7 +14236,7 @@
         <v>7.747999999999999</v>
       </c>
       <c r="P206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q206" t="n">
         <v>1.046042665095654</v>
@@ -14294,16 +14294,16 @@
         <v>9.26</v>
       </c>
       <c r="M207" t="n">
-        <v>7.43</v>
+        <v>6.81</v>
       </c>
       <c r="N207" t="n">
         <v>3.48</v>
       </c>
       <c r="O207" t="n">
-        <v>7.847</v>
+        <v>7.723</v>
       </c>
       <c r="P207" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q207" t="n">
         <v>1.743404441826089</v>
@@ -14361,13 +14361,13 @@
         <v>8.15</v>
       </c>
       <c r="M208" t="n">
-        <v>9.960000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="N208" t="n">
         <v>4.64</v>
       </c>
       <c r="O208" t="n">
-        <v>7.6975</v>
+        <v>7.4915</v>
       </c>
       <c r="P208" t="n">
         <v>3</v>
@@ -14495,13 +14495,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M210" t="n">
-        <v>7.43</v>
+        <v>7.28</v>
       </c>
       <c r="N210" t="n">
         <v>3.48</v>
       </c>
       <c r="O210" t="n">
-        <v>8.237499999999999</v>
+        <v>8.2075</v>
       </c>
       <c r="P210" t="n">
         <v>2</v>
@@ -14562,13 +14562,13 @@
         <v>9.039999999999999</v>
       </c>
       <c r="M211" t="n">
-        <v>9.32</v>
+        <v>9.08</v>
       </c>
       <c r="N211" t="n">
         <v>6.37</v>
       </c>
       <c r="O211" t="n">
-        <v>8.653499999999999</v>
+        <v>8.605499999999999</v>
       </c>
       <c r="P211" t="n">
         <v>1</v>
@@ -14629,13 +14629,13 @@
         <v>10</v>
       </c>
       <c r="M212" t="n">
-        <v>4.33</v>
+        <v>3.85</v>
       </c>
       <c r="N212" t="n">
         <v>2.86</v>
       </c>
       <c r="O212" t="n">
-        <v>7.744</v>
+        <v>7.648</v>
       </c>
       <c r="P212" t="n">
         <v>3</v>
@@ -14696,13 +14696,13 @@
         <v>9.779999999999999</v>
       </c>
       <c r="M213" t="n">
-        <v>6.79</v>
+        <v>5.6</v>
       </c>
       <c r="N213" t="n">
         <v>5.01</v>
       </c>
       <c r="O213" t="n">
-        <v>8.2895</v>
+        <v>8.051499999999999</v>
       </c>
       <c r="P213" t="n">
         <v>2</v>
@@ -14763,13 +14763,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M214" t="n">
-        <v>8.140000000000001</v>
+        <v>8.43</v>
       </c>
       <c r="N214" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O214" t="n">
-        <v>8.379999999999999</v>
+        <v>8.437999999999999</v>
       </c>
       <c r="P214" t="n">
         <v>1</v>
@@ -14830,13 +14830,13 @@
         <v>9.93</v>
       </c>
       <c r="M215" t="n">
-        <v>6.34</v>
+        <v>5.98</v>
       </c>
       <c r="N215" t="n">
         <v>2.86</v>
       </c>
       <c r="O215" t="n">
-        <v>8.022499999999999</v>
+        <v>7.9505</v>
       </c>
       <c r="P215" t="n">
         <v>3</v>
@@ -14897,16 +14897,16 @@
         <v>9.33</v>
       </c>
       <c r="M216" t="n">
-        <v>8.42</v>
+        <v>7.5</v>
       </c>
       <c r="N216" t="n">
         <v>5.01</v>
       </c>
       <c r="O216" t="n">
-        <v>8.308</v>
+        <v>8.123999999999999</v>
       </c>
       <c r="P216" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q216" t="n">
         <v>1.718101934882773</v>
@@ -14964,16 +14964,16 @@
         <v>8.15</v>
       </c>
       <c r="M217" t="n">
-        <v>9.59</v>
+        <v>9.99</v>
       </c>
       <c r="N217" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O217" t="n">
-        <v>8.161999999999999</v>
+        <v>8.241999999999999</v>
       </c>
       <c r="P217" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q217" t="n">
         <v>2.863503224804621</v>
@@ -15098,13 +15098,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M219" t="n">
-        <v>7.43</v>
+        <v>6.88</v>
       </c>
       <c r="N219" t="n">
         <v>3.48</v>
       </c>
       <c r="O219" t="n">
-        <v>8.144499999999999</v>
+        <v>8.0345</v>
       </c>
       <c r="P219" t="n">
         <v>2</v>
@@ -15165,13 +15165,13 @@
         <v>8.74</v>
       </c>
       <c r="M220" t="n">
-        <v>9.960000000000001</v>
+        <v>9.07</v>
       </c>
       <c r="N220" t="n">
         <v>7.6</v>
       </c>
       <c r="O220" t="n">
-        <v>8.615</v>
+        <v>8.436999999999999</v>
       </c>
       <c r="P220" t="n">
         <v>1</v>
@@ -15241,7 +15241,7 @@
         <v>7.747999999999999</v>
       </c>
       <c r="P221" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q221" t="n">
         <v>1.046042665095654</v>
@@ -15299,16 +15299,16 @@
         <v>9.26</v>
       </c>
       <c r="M222" t="n">
-        <v>7.43</v>
+        <v>6.81</v>
       </c>
       <c r="N222" t="n">
         <v>3.48</v>
       </c>
       <c r="O222" t="n">
-        <v>7.847</v>
+        <v>7.723</v>
       </c>
       <c r="P222" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q222" t="n">
         <v>1.743404441826089</v>
@@ -15366,13 +15366,13 @@
         <v>8.15</v>
       </c>
       <c r="M223" t="n">
-        <v>9.960000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="N223" t="n">
         <v>4.64</v>
       </c>
       <c r="O223" t="n">
-        <v>7.6975</v>
+        <v>7.4915</v>
       </c>
       <c r="P223" t="n">
         <v>3</v>
@@ -15500,13 +15500,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M225" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N225" t="n">
         <v>3.48</v>
       </c>
       <c r="O225" t="n">
-        <v>8.054499999999999</v>
+        <v>7.9085</v>
       </c>
       <c r="P225" t="n">
         <v>2</v>
@@ -15567,13 +15567,13 @@
         <v>8.74</v>
       </c>
       <c r="M226" t="n">
-        <v>9.960000000000001</v>
+        <v>8.69</v>
       </c>
       <c r="N226" t="n">
         <v>7.6</v>
       </c>
       <c r="O226" t="n">
-        <v>8.474</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="P226" t="n">
         <v>1</v>
@@ -15643,7 +15643,7 @@
         <v>7.795999999999999</v>
       </c>
       <c r="P227" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Q227" t="n">
         <v>0.9349584882713364</v>
@@ -15701,13 +15701,13 @@
         <v>9.26</v>
       </c>
       <c r="M228" t="n">
-        <v>7.43</v>
+        <v>7.04</v>
       </c>
       <c r="N228" t="n">
         <v>3.48</v>
       </c>
       <c r="O228" t="n">
-        <v>7.925</v>
+        <v>7.847</v>
       </c>
       <c r="P228" t="n">
         <v>1</v>
@@ -15768,16 +15768,16 @@
         <v>8.15</v>
       </c>
       <c r="M229" t="n">
-        <v>9.960000000000001</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="N229" t="n">
         <v>4.64</v>
       </c>
       <c r="O229" t="n">
-        <v>7.8205</v>
+        <v>7.7065</v>
       </c>
       <c r="P229" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q229" t="n">
         <v>2.49322263539023</v>
@@ -15902,13 +15902,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M231" t="n">
-        <v>7.43</v>
+        <v>6.72</v>
       </c>
       <c r="N231" t="n">
         <v>3.48</v>
       </c>
       <c r="O231" t="n">
-        <v>8.090499999999999</v>
+        <v>7.9485</v>
       </c>
       <c r="P231" t="n">
         <v>2</v>
@@ -15969,13 +15969,13 @@
         <v>8.74</v>
       </c>
       <c r="M232" t="n">
-        <v>9.960000000000001</v>
+        <v>8.74</v>
       </c>
       <c r="N232" t="n">
         <v>7.6</v>
       </c>
       <c r="O232" t="n">
-        <v>8.530999999999999</v>
+        <v>8.286999999999999</v>
       </c>
       <c r="P232" t="n">
         <v>1</v>
@@ -16036,13 +16036,13 @@
         <v>9.039999999999999</v>
       </c>
       <c r="M233" t="n">
-        <v>6.34</v>
+        <v>5.94</v>
       </c>
       <c r="N233" t="n">
         <v>1.51</v>
       </c>
       <c r="O233" t="n">
-        <v>7.049499999999999</v>
+        <v>6.9695</v>
       </c>
       <c r="P233" t="n">
         <v>1</v>
@@ -16103,13 +16103,13 @@
         <v>8</v>
       </c>
       <c r="M234" t="n">
-        <v>8.42</v>
+        <v>7.4</v>
       </c>
       <c r="N234" t="n">
         <v>1.51</v>
       </c>
       <c r="O234" t="n">
-        <v>6.6335</v>
+        <v>6.4295</v>
       </c>
       <c r="P234" t="n">
         <v>2</v>
@@ -16170,13 +16170,13 @@
         <v>6.96</v>
       </c>
       <c r="M235" t="n">
-        <v>9.9</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="N235" t="n">
         <v>4.64</v>
       </c>
       <c r="O235" t="n">
-        <v>6.564</v>
+        <v>6.308</v>
       </c>
       <c r="P235" t="n">
         <v>3</v>
@@ -16438,16 +16438,16 @@
         <v>9.26</v>
       </c>
       <c r="M239" t="n">
-        <v>7.43</v>
+        <v>6.7</v>
       </c>
       <c r="N239" t="n">
         <v>1.51</v>
       </c>
       <c r="O239" t="n">
-        <v>7.4975</v>
+        <v>7.3515</v>
       </c>
       <c r="P239" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q239" t="n">
         <v>1.86683130496422</v>
@@ -16505,16 +16505,16 @@
         <v>8.15</v>
       </c>
       <c r="M240" t="n">
-        <v>9.9</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="N240" t="n">
         <v>4.64</v>
       </c>
       <c r="O240" t="n">
-        <v>7.6015</v>
+        <v>7.345499999999999</v>
       </c>
       <c r="P240" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q240" t="n">
         <v>2.986930087942751</v>
@@ -16572,13 +16572,13 @@
         <v>6.67</v>
       </c>
       <c r="M241" t="n">
-        <v>7.62</v>
+        <v>7.97</v>
       </c>
       <c r="N241" t="n">
         <v>6.69</v>
       </c>
       <c r="O241" t="n">
-        <v>6.305</v>
+        <v>6.375</v>
       </c>
       <c r="P241" t="n">
         <v>3</v>

</xml_diff>

<commit_message>
modified shower and appliance formulas, hybrid prompt and reran al gt and rag. also updated paper_working_draft accordingly
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_shower.xlsx
+++ b/Ground Truth/ground_truth_shower.xlsx
@@ -1162,13 +1162,13 @@
         <v>9.26</v>
       </c>
       <c r="M11" t="n">
-        <v>7.43</v>
+        <v>7.37</v>
       </c>
       <c r="N11" t="n">
         <v>3.48</v>
       </c>
       <c r="O11" t="n">
-        <v>8.020999999999999</v>
+        <v>8.009</v>
       </c>
       <c r="P11" t="n">
         <v>2</v>
@@ -1229,13 +1229,13 @@
         <v>8.52</v>
       </c>
       <c r="M12" t="n">
-        <v>9.32</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="N12" t="n">
         <v>6.37</v>
       </c>
       <c r="O12" t="n">
-        <v>8.3515</v>
+        <v>8.3315</v>
       </c>
       <c r="P12" t="n">
         <v>1</v>
@@ -1296,13 +1296,13 @@
         <v>7.41</v>
       </c>
       <c r="M13" t="n">
-        <v>9.59</v>
+        <v>9.609999999999999</v>
       </c>
       <c r="N13" t="n">
         <v>5.71</v>
       </c>
       <c r="O13" t="n">
-        <v>7.581999999999999</v>
+        <v>7.585999999999999</v>
       </c>
       <c r="P13" t="n">
         <v>3</v>
@@ -5182,13 +5182,13 @@
         <v>9.039999999999999</v>
       </c>
       <c r="M71" t="n">
-        <v>6.26</v>
+        <v>6.23</v>
       </c>
       <c r="N71" t="n">
         <v>2.86</v>
       </c>
       <c r="O71" t="n">
-        <v>7.515</v>
+        <v>7.509</v>
       </c>
       <c r="P71" t="n">
         <v>1</v>
@@ -5249,13 +5249,13 @@
         <v>7.48</v>
       </c>
       <c r="M72" t="n">
-        <v>9.08</v>
+        <v>8.99</v>
       </c>
       <c r="N72" t="n">
         <v>3.07</v>
       </c>
       <c r="O72" t="n">
-        <v>7.0665</v>
+        <v>7.0485</v>
       </c>
       <c r="P72" t="n">
         <v>2</v>
@@ -5316,13 +5316,13 @@
         <v>5.93</v>
       </c>
       <c r="M73" t="n">
-        <v>9.640000000000001</v>
+        <v>9.66</v>
       </c>
       <c r="N73" t="n">
         <v>5.71</v>
       </c>
       <c r="O73" t="n">
-        <v>6.534</v>
+        <v>6.537999999999999</v>
       </c>
       <c r="P73" t="n">
         <v>3</v>
@@ -5383,13 +5383,13 @@
         <v>8.74</v>
       </c>
       <c r="M74" t="n">
-        <v>6.07</v>
+        <v>6.05</v>
       </c>
       <c r="N74" t="n">
         <v>2.86</v>
       </c>
       <c r="O74" t="n">
-        <v>7.15</v>
+        <v>7.146</v>
       </c>
       <c r="P74" t="n">
         <v>1</v>
@@ -5450,13 +5450,13 @@
         <v>6.96</v>
       </c>
       <c r="M75" t="n">
-        <v>8.49</v>
+        <v>8.42</v>
       </c>
       <c r="N75" t="n">
         <v>3.07</v>
       </c>
       <c r="O75" t="n">
-        <v>6.3825</v>
+        <v>6.3685</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
@@ -5517,13 +5517,13 @@
         <v>5.19</v>
       </c>
       <c r="M76" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="N76" t="n">
         <v>5.71</v>
       </c>
       <c r="O76" t="n">
-        <v>5.611999999999999</v>
+        <v>5.617999999999999</v>
       </c>
       <c r="P76" t="n">
         <v>3</v>
@@ -5651,13 +5651,13 @@
         <v>8.74</v>
       </c>
       <c r="M78" t="n">
-        <v>9.24</v>
+        <v>9.16</v>
       </c>
       <c r="N78" t="n">
         <v>4.64</v>
       </c>
       <c r="O78" t="n">
-        <v>8.077999999999999</v>
+        <v>8.061999999999999</v>
       </c>
       <c r="P78" t="n">
         <v>1</v>
@@ -5785,13 +5785,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M80" t="n">
-        <v>6.19</v>
+        <v>6.16</v>
       </c>
       <c r="N80" t="n">
         <v>2.86</v>
       </c>
       <c r="O80" t="n">
-        <v>7.869500000000001</v>
+        <v>7.863500000000001</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -5852,13 +5852,13 @@
         <v>7.41</v>
       </c>
       <c r="M81" t="n">
-        <v>9.699999999999999</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="N81" t="n">
         <v>5.71</v>
       </c>
       <c r="O81" t="n">
-        <v>7.471999999999999</v>
+        <v>7.475999999999999</v>
       </c>
       <c r="P81" t="n">
         <v>2</v>
@@ -5986,13 +5986,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M83" t="n">
-        <v>6.85</v>
+        <v>6.81</v>
       </c>
       <c r="N83" t="n">
         <v>3.48</v>
       </c>
       <c r="O83" t="n">
-        <v>8.016500000000001</v>
+        <v>8.0085</v>
       </c>
       <c r="P83" t="n">
         <v>1</v>
@@ -6053,13 +6053,13 @@
         <v>7.56</v>
       </c>
       <c r="M84" t="n">
-        <v>7.84</v>
+        <v>7.87</v>
       </c>
       <c r="N84" t="n">
         <v>6.69</v>
       </c>
       <c r="O84" t="n">
-        <v>7.161499999999999</v>
+        <v>7.1675</v>
       </c>
       <c r="P84" t="n">
         <v>2</v>
@@ -6388,13 +6388,13 @@
         <v>9.33</v>
       </c>
       <c r="M89" t="n">
-        <v>8.289999999999999</v>
+        <v>8.220000000000001</v>
       </c>
       <c r="N89" t="n">
         <v>5.01</v>
       </c>
       <c r="O89" t="n">
-        <v>8.452999999999999</v>
+        <v>8.439</v>
       </c>
       <c r="P89" t="n">
         <v>1</v>
@@ -6455,13 +6455,13 @@
         <v>8.15</v>
       </c>
       <c r="M90" t="n">
-        <v>9.619999999999999</v>
+        <v>9.640000000000001</v>
       </c>
       <c r="N90" t="n">
         <v>5.71</v>
       </c>
       <c r="O90" t="n">
-        <v>8.039</v>
+        <v>8.042999999999999</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
@@ -6589,13 +6589,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M92" t="n">
-        <v>4.98</v>
+        <v>4.94</v>
       </c>
       <c r="N92" t="n">
         <v>3.48</v>
       </c>
       <c r="O92" t="n">
-        <v>7.654500000000001</v>
+        <v>7.646500000000001</v>
       </c>
       <c r="P92" t="n">
         <v>2</v>
@@ -6656,13 +6656,13 @@
         <v>8.74</v>
       </c>
       <c r="M93" t="n">
-        <v>7.55</v>
+        <v>7.46</v>
       </c>
       <c r="N93" t="n">
         <v>7.6</v>
       </c>
       <c r="O93" t="n">
-        <v>8.132999999999999</v>
+        <v>8.115</v>
       </c>
       <c r="P93" t="n">
         <v>1</v>
@@ -6723,13 +6723,13 @@
         <v>7.56</v>
       </c>
       <c r="M94" t="n">
-        <v>7.9</v>
+        <v>7.92</v>
       </c>
       <c r="N94" t="n">
         <v>6.69</v>
       </c>
       <c r="O94" t="n">
-        <v>7.2005</v>
+        <v>7.2045</v>
       </c>
       <c r="P94" t="n">
         <v>3</v>
@@ -6790,13 +6790,13 @@
         <v>9.26</v>
       </c>
       <c r="M95" t="n">
-        <v>4.84</v>
+        <v>4.8</v>
       </c>
       <c r="N95" t="n">
         <v>3.48</v>
       </c>
       <c r="O95" t="n">
-        <v>7.308</v>
+        <v>7.3</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
@@ -6857,13 +6857,13 @@
         <v>8.15</v>
       </c>
       <c r="M96" t="n">
-        <v>7.27</v>
+        <v>7.19</v>
       </c>
       <c r="N96" t="n">
         <v>4.64</v>
       </c>
       <c r="O96" t="n">
-        <v>7.126499999999999</v>
+        <v>7.1105</v>
       </c>
       <c r="P96" t="n">
         <v>2</v>
@@ -6924,13 +6924,13 @@
         <v>6.67</v>
       </c>
       <c r="M97" t="n">
-        <v>7.99</v>
+        <v>8.01</v>
       </c>
       <c r="N97" t="n">
         <v>6.69</v>
       </c>
       <c r="O97" t="n">
-        <v>6.457</v>
+        <v>6.461</v>
       </c>
       <c r="P97" t="n">
         <v>3</v>
@@ -6991,13 +6991,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M98" t="n">
-        <v>7.04</v>
+        <v>7</v>
       </c>
       <c r="N98" t="n">
         <v>3.48</v>
       </c>
       <c r="O98" t="n">
-        <v>8.108499999999999</v>
+        <v>8.1005</v>
       </c>
       <c r="P98" t="n">
         <v>2</v>
@@ -7058,13 +7058,13 @@
         <v>8.74</v>
       </c>
       <c r="M99" t="n">
-        <v>9.390000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="N99" t="n">
         <v>7.6</v>
       </c>
       <c r="O99" t="n">
-        <v>8.567</v>
+        <v>8.551</v>
       </c>
       <c r="P99" t="n">
         <v>1</v>
@@ -7125,13 +7125,13 @@
         <v>7.56</v>
       </c>
       <c r="M100" t="n">
-        <v>9.31</v>
+        <v>9.33</v>
       </c>
       <c r="N100" t="n">
         <v>6.69</v>
       </c>
       <c r="O100" t="n">
-        <v>7.581499999999999</v>
+        <v>7.585499999999999</v>
       </c>
       <c r="P100" t="n">
         <v>3</v>
@@ -7192,13 +7192,13 @@
         <v>9.26</v>
       </c>
       <c r="M101" t="n">
-        <v>6.94</v>
+        <v>6.9</v>
       </c>
       <c r="N101" t="n">
         <v>3.48</v>
       </c>
       <c r="O101" t="n">
-        <v>7.794</v>
+        <v>7.786</v>
       </c>
       <c r="P101" t="n">
         <v>2</v>
@@ -7259,13 +7259,13 @@
         <v>8.15</v>
       </c>
       <c r="M102" t="n">
-        <v>9.19</v>
+        <v>9.109999999999999</v>
       </c>
       <c r="N102" t="n">
         <v>7.6</v>
       </c>
       <c r="O102" t="n">
-        <v>8.0595</v>
+        <v>8.0435</v>
       </c>
       <c r="P102" t="n">
         <v>1</v>
@@ -7326,13 +7326,13 @@
         <v>6.67</v>
       </c>
       <c r="M103" t="n">
-        <v>9.35</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="N103" t="n">
         <v>6.69</v>
       </c>
       <c r="O103" t="n">
-        <v>6.885</v>
+        <v>6.888999999999999</v>
       </c>
       <c r="P103" t="n">
         <v>3</v>
@@ -7393,13 +7393,13 @@
         <v>9.26</v>
       </c>
       <c r="M104" t="n">
-        <v>5.9</v>
+        <v>5.86</v>
       </c>
       <c r="N104" t="n">
         <v>3.48</v>
       </c>
       <c r="O104" t="n">
-        <v>7.541</v>
+        <v>7.532999999999999</v>
       </c>
       <c r="P104" t="n">
         <v>1</v>
@@ -7460,13 +7460,13 @@
         <v>8.15</v>
       </c>
       <c r="M105" t="n">
-        <v>8.109999999999999</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="N105" t="n">
         <v>4.64</v>
       </c>
       <c r="O105" t="n">
-        <v>7.3275</v>
+        <v>7.3115</v>
       </c>
       <c r="P105" t="n">
         <v>2</v>
@@ -7527,13 +7527,13 @@
         <v>6.67</v>
       </c>
       <c r="M106" t="n">
-        <v>7.04</v>
+        <v>7.07</v>
       </c>
       <c r="N106" t="n">
         <v>6.69</v>
       </c>
       <c r="O106" t="n">
-        <v>6.311999999999999</v>
+        <v>6.318</v>
       </c>
       <c r="P106" t="n">
         <v>3</v>
@@ -7594,13 +7594,13 @@
         <v>8.15</v>
       </c>
       <c r="M107" t="n">
-        <v>9.119999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="N107" t="n">
         <v>4.64</v>
       </c>
       <c r="O107" t="n">
-        <v>7.6015</v>
+        <v>7.5855</v>
       </c>
       <c r="P107" t="n">
         <v>1</v>
@@ -7661,13 +7661,13 @@
         <v>7.41</v>
       </c>
       <c r="M108" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="N108" t="n">
         <v>5.71</v>
       </c>
       <c r="O108" t="n">
-        <v>7.217</v>
+        <v>7.223</v>
       </c>
       <c r="P108" t="n">
         <v>2</v>
@@ -7728,13 +7728,13 @@
         <v>6.67</v>
       </c>
       <c r="M109" t="n">
-        <v>7.79</v>
+        <v>7.81</v>
       </c>
       <c r="N109" t="n">
         <v>6.69</v>
       </c>
       <c r="O109" t="n">
-        <v>6.573</v>
+        <v>6.577</v>
       </c>
       <c r="P109" t="n">
         <v>3</v>
@@ -7795,13 +7795,13 @@
         <v>7.56</v>
       </c>
       <c r="M110" t="n">
-        <v>8.93</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="N110" t="n">
         <v>4.64</v>
       </c>
       <c r="O110" t="n">
-        <v>7.071999999999999</v>
+        <v>7.058</v>
       </c>
       <c r="P110" t="n">
         <v>1</v>
@@ -7862,13 +7862,13 @@
         <v>6.67</v>
       </c>
       <c r="M111" t="n">
-        <v>9.15</v>
+        <v>9.19</v>
       </c>
       <c r="N111" t="n">
         <v>5.71</v>
       </c>
       <c r="O111" t="n">
-        <v>6.619999999999999</v>
+        <v>6.627999999999999</v>
       </c>
       <c r="P111" t="n">
         <v>2</v>
@@ -7929,13 +7929,13 @@
         <v>5.78</v>
       </c>
       <c r="M112" t="n">
-        <v>7.84</v>
+        <v>7.87</v>
       </c>
       <c r="N112" t="n">
         <v>6.69</v>
       </c>
       <c r="O112" t="n">
-        <v>5.8455</v>
+        <v>5.8515</v>
       </c>
       <c r="P112" t="n">
         <v>3</v>
@@ -7996,13 +7996,13 @@
         <v>8.15</v>
       </c>
       <c r="M113" t="n">
-        <v>9.32</v>
+        <v>9.24</v>
       </c>
       <c r="N113" t="n">
         <v>4.64</v>
       </c>
       <c r="O113" t="n">
-        <v>7.6925</v>
+        <v>7.6765</v>
       </c>
       <c r="P113" t="n">
         <v>1</v>
@@ -8063,13 +8063,13 @@
         <v>7.41</v>
       </c>
       <c r="M114" t="n">
-        <v>9</v>
+        <v>9.02</v>
       </c>
       <c r="N114" t="n">
         <v>5.71</v>
       </c>
       <c r="O114" t="n">
-        <v>7.265999999999999</v>
+        <v>7.27</v>
       </c>
       <c r="P114" t="n">
         <v>2</v>
@@ -8130,13 +8130,13 @@
         <v>6.67</v>
       </c>
       <c r="M115" t="n">
-        <v>7.74</v>
+        <v>7.76</v>
       </c>
       <c r="N115" t="n">
         <v>6.69</v>
       </c>
       <c r="O115" t="n">
-        <v>6.640999999999999</v>
+        <v>6.644999999999999</v>
       </c>
       <c r="P115" t="n">
         <v>3</v>
@@ -8197,13 +8197,13 @@
         <v>8.74</v>
       </c>
       <c r="M116" t="n">
-        <v>9.119999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="N116" t="n">
         <v>4.64</v>
       </c>
       <c r="O116" t="n">
-        <v>8.026999999999999</v>
+        <v>8.010999999999999</v>
       </c>
       <c r="P116" t="n">
         <v>1</v>
@@ -8264,13 +8264,13 @@
         <v>8.15</v>
       </c>
       <c r="M117" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="N117" t="n">
         <v>5.71</v>
       </c>
       <c r="O117" t="n">
-        <v>7.752</v>
+        <v>7.758</v>
       </c>
       <c r="P117" t="n">
         <v>2</v>
@@ -8331,13 +8331,13 @@
         <v>7.56</v>
       </c>
       <c r="M118" t="n">
-        <v>7.79</v>
+        <v>7.81</v>
       </c>
       <c r="N118" t="n">
         <v>6.69</v>
       </c>
       <c r="O118" t="n">
-        <v>7.2145</v>
+        <v>7.218500000000001</v>
       </c>
       <c r="P118" t="n">
         <v>3</v>
@@ -8398,13 +8398,13 @@
         <v>8.15</v>
       </c>
       <c r="M119" t="n">
-        <v>9.24</v>
+        <v>9.16</v>
       </c>
       <c r="N119" t="n">
         <v>4.64</v>
       </c>
       <c r="O119" t="n">
-        <v>7.655499999999999</v>
+        <v>7.639499999999999</v>
       </c>
       <c r="P119" t="n">
         <v>1</v>
@@ -8465,13 +8465,13 @@
         <v>7.41</v>
       </c>
       <c r="M120" t="n">
-        <v>9.02</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="N120" t="n">
         <v>5.71</v>
       </c>
       <c r="O120" t="n">
-        <v>7.246</v>
+        <v>7.252</v>
       </c>
       <c r="P120" t="n">
         <v>2</v>
@@ -8532,13 +8532,13 @@
         <v>6.67</v>
       </c>
       <c r="M121" t="n">
-        <v>7.76</v>
+        <v>7.78</v>
       </c>
       <c r="N121" t="n">
         <v>6.69</v>
       </c>
       <c r="O121" t="n">
-        <v>6.611999999999999</v>
+        <v>6.616</v>
       </c>
       <c r="P121" t="n">
         <v>3</v>
@@ -9202,13 +9202,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M131" t="n">
-        <v>7.43</v>
+        <v>7.37</v>
       </c>
       <c r="N131" t="n">
         <v>3.48</v>
       </c>
       <c r="O131" t="n">
-        <v>8.2645</v>
+        <v>8.2525</v>
       </c>
       <c r="P131" t="n">
         <v>2</v>
@@ -9269,13 +9269,13 @@
         <v>8.74</v>
       </c>
       <c r="M132" t="n">
-        <v>9.960000000000001</v>
+        <v>9.99</v>
       </c>
       <c r="N132" t="n">
         <v>7.6</v>
       </c>
       <c r="O132" t="n">
-        <v>8.807</v>
+        <v>8.813000000000001</v>
       </c>
       <c r="P132" t="n">
         <v>1</v>
@@ -9336,13 +9336,13 @@
         <v>7.56</v>
       </c>
       <c r="M133" t="n">
-        <v>9.210000000000001</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="N133" t="n">
         <v>6.69</v>
       </c>
       <c r="O133" t="n">
-        <v>7.7505</v>
+        <v>7.7525</v>
       </c>
       <c r="P133" t="n">
         <v>3</v>
@@ -9604,13 +9604,13 @@
         <v>9.33</v>
       </c>
       <c r="M137" t="n">
-        <v>5.95</v>
+        <v>5.94</v>
       </c>
       <c r="N137" t="n">
         <v>2.86</v>
       </c>
       <c r="O137" t="n">
-        <v>7.4735</v>
+        <v>7.471500000000001</v>
       </c>
       <c r="P137" t="n">
         <v>1</v>
@@ -9671,13 +9671,13 @@
         <v>8</v>
       </c>
       <c r="M138" t="n">
-        <v>8.1</v>
+        <v>8.07</v>
       </c>
       <c r="N138" t="n">
         <v>3.07</v>
       </c>
       <c r="O138" t="n">
-        <v>6.911499999999999</v>
+        <v>6.905499999999999</v>
       </c>
       <c r="P138" t="n">
         <v>2</v>
@@ -9738,13 +9738,13 @@
         <v>6.67</v>
       </c>
       <c r="M139" t="n">
-        <v>9.9</v>
+        <v>9.85</v>
       </c>
       <c r="N139" t="n">
         <v>5.71</v>
       </c>
       <c r="O139" t="n">
-        <v>6.644</v>
+        <v>6.633999999999999</v>
       </c>
       <c r="P139" t="n">
         <v>3</v>
@@ -10073,13 +10073,13 @@
         <v>9.33</v>
       </c>
       <c r="M144" t="n">
-        <v>7.74</v>
+        <v>7.69</v>
       </c>
       <c r="N144" t="n">
         <v>5.01</v>
       </c>
       <c r="O144" t="n">
-        <v>8.234999999999999</v>
+        <v>8.225</v>
       </c>
       <c r="P144" t="n">
         <v>1</v>
@@ -10140,13 +10140,13 @@
         <v>7.56</v>
       </c>
       <c r="M145" t="n">
-        <v>9.35</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="N145" t="n">
         <v>6.69</v>
       </c>
       <c r="O145" t="n">
-        <v>7.5265</v>
+        <v>7.5305</v>
       </c>
       <c r="P145" t="n">
         <v>2</v>
@@ -10207,13 +10207,13 @@
         <v>8.52</v>
       </c>
       <c r="M146" t="n">
-        <v>8.74</v>
+        <v>8.66</v>
       </c>
       <c r="N146" t="n">
         <v>6.37</v>
       </c>
       <c r="O146" t="n">
-        <v>8.115499999999999</v>
+        <v>8.099499999999999</v>
       </c>
       <c r="P146" t="n">
         <v>1</v>
@@ -10274,13 +10274,13 @@
         <v>5.93</v>
       </c>
       <c r="M147" t="n">
-        <v>8.84</v>
+        <v>8.85</v>
       </c>
       <c r="N147" t="n">
         <v>5.71</v>
       </c>
       <c r="O147" t="n">
-        <v>6.226999999999999</v>
+        <v>6.229</v>
       </c>
       <c r="P147" t="n">
         <v>2</v>
@@ -10408,13 +10408,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M149" t="n">
-        <v>4.94</v>
+        <v>4.9</v>
       </c>
       <c r="N149" t="n">
         <v>3.48</v>
       </c>
       <c r="O149" t="n">
-        <v>7.634500000000001</v>
+        <v>7.626500000000001</v>
       </c>
       <c r="P149" t="n">
         <v>2</v>
@@ -10475,13 +10475,13 @@
         <v>8.74</v>
       </c>
       <c r="M150" t="n">
-        <v>7.46</v>
+        <v>7.38</v>
       </c>
       <c r="N150" t="n">
         <v>4.64</v>
       </c>
       <c r="O150" t="n">
-        <v>7.656</v>
+        <v>7.64</v>
       </c>
       <c r="P150" t="n">
         <v>1</v>
@@ -10542,13 +10542,13 @@
         <v>7.56</v>
       </c>
       <c r="M151" t="n">
-        <v>7.92</v>
+        <v>7.95</v>
       </c>
       <c r="N151" t="n">
         <v>6.69</v>
       </c>
       <c r="O151" t="n">
-        <v>7.177499999999999</v>
+        <v>7.1835</v>
       </c>
       <c r="P151" t="n">
         <v>3</v>
@@ -10609,13 +10609,13 @@
         <v>9.26</v>
       </c>
       <c r="M152" t="n">
-        <v>6.1</v>
+        <v>6.06</v>
       </c>
       <c r="N152" t="n">
         <v>3.48</v>
       </c>
       <c r="O152" t="n">
-        <v>7.643999999999999</v>
+        <v>7.635999999999999</v>
       </c>
       <c r="P152" t="n">
         <v>2</v>
@@ -10676,13 +10676,13 @@
         <v>8.15</v>
       </c>
       <c r="M153" t="n">
-        <v>8.59</v>
+        <v>8.5</v>
       </c>
       <c r="N153" t="n">
         <v>7.6</v>
       </c>
       <c r="O153" t="n">
-        <v>7.969499999999999</v>
+        <v>7.951499999999999</v>
       </c>
       <c r="P153" t="n">
         <v>1</v>
@@ -10743,13 +10743,13 @@
         <v>6.67</v>
       </c>
       <c r="M154" t="n">
-        <v>8.609999999999999</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="N154" t="n">
         <v>6.69</v>
       </c>
       <c r="O154" t="n">
-        <v>6.781999999999999</v>
+        <v>6.786</v>
       </c>
       <c r="P154" t="n">
         <v>3</v>
@@ -10810,13 +10810,13 @@
         <v>8.890000000000001</v>
       </c>
       <c r="M155" t="n">
-        <v>7.74</v>
+        <v>7.69</v>
       </c>
       <c r="N155" t="n">
         <v>1.51</v>
       </c>
       <c r="O155" t="n">
-        <v>7.391</v>
+        <v>7.381</v>
       </c>
       <c r="P155" t="n">
         <v>2</v>
@@ -10877,13 +10877,13 @@
         <v>8.15</v>
       </c>
       <c r="M156" t="n">
-        <v>9.119999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="N156" t="n">
         <v>4.64</v>
       </c>
       <c r="O156" t="n">
-        <v>7.6015</v>
+        <v>7.5855</v>
       </c>
       <c r="P156" t="n">
         <v>1</v>
@@ -10944,13 +10944,13 @@
         <v>7.41</v>
       </c>
       <c r="M157" t="n">
-        <v>9.07</v>
+        <v>9.1</v>
       </c>
       <c r="N157" t="n">
         <v>5.71</v>
       </c>
       <c r="O157" t="n">
-        <v>7.217</v>
+        <v>7.223</v>
       </c>
       <c r="P157" t="n">
         <v>3</v>
@@ -11011,13 +11011,13 @@
         <v>8.15</v>
       </c>
       <c r="M158" t="n">
-        <v>9.24</v>
+        <v>9.16</v>
       </c>
       <c r="N158" t="n">
         <v>4.64</v>
       </c>
       <c r="O158" t="n">
-        <v>7.655499999999999</v>
+        <v>7.639499999999999</v>
       </c>
       <c r="P158" t="n">
         <v>1</v>
@@ -11078,13 +11078,13 @@
         <v>7.41</v>
       </c>
       <c r="M159" t="n">
-        <v>9.02</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="N159" t="n">
         <v>5.71</v>
       </c>
       <c r="O159" t="n">
-        <v>7.246</v>
+        <v>7.252</v>
       </c>
       <c r="P159" t="n">
         <v>2</v>
@@ -11145,13 +11145,13 @@
         <v>6.67</v>
       </c>
       <c r="M160" t="n">
-        <v>7.76</v>
+        <v>7.78</v>
       </c>
       <c r="N160" t="n">
         <v>6.69</v>
       </c>
       <c r="O160" t="n">
-        <v>6.611999999999999</v>
+        <v>6.616</v>
       </c>
       <c r="P160" t="n">
         <v>3</v>
@@ -11681,13 +11681,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M168" t="n">
-        <v>7.15</v>
+        <v>7.11</v>
       </c>
       <c r="N168" t="n">
         <v>3.48</v>
       </c>
       <c r="O168" t="n">
-        <v>8.154500000000001</v>
+        <v>8.146500000000001</v>
       </c>
       <c r="P168" t="n">
         <v>2</v>
@@ -11748,13 +11748,13 @@
         <v>8.74</v>
       </c>
       <c r="M169" t="n">
-        <v>9.619999999999999</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="N169" t="n">
         <v>7.6</v>
       </c>
       <c r="O169" t="n">
-        <v>8.654999999999999</v>
+        <v>8.636999999999999</v>
       </c>
       <c r="P169" t="n">
         <v>1</v>
@@ -12083,13 +12083,13 @@
         <v>9.26</v>
       </c>
       <c r="M174" t="n">
-        <v>7.34</v>
+        <v>7.28</v>
       </c>
       <c r="N174" t="n">
         <v>3.48</v>
       </c>
       <c r="O174" t="n">
-        <v>7.984999999999999</v>
+        <v>7.973</v>
       </c>
       <c r="P174" t="n">
         <v>1</v>
@@ -12150,13 +12150,13 @@
         <v>8.15</v>
       </c>
       <c r="M175" t="n">
-        <v>9.99</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="N175" t="n">
         <v>4.64</v>
       </c>
       <c r="O175" t="n">
-        <v>7.9525</v>
+        <v>7.930499999999999</v>
       </c>
       <c r="P175" t="n">
         <v>2</v>
@@ -12284,13 +12284,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M177" t="n">
-        <v>7</v>
+        <v>6.96</v>
       </c>
       <c r="N177" t="n">
         <v>3.48</v>
       </c>
       <c r="O177" t="n">
-        <v>8.0885</v>
+        <v>8.080500000000001</v>
       </c>
       <c r="P177" t="n">
         <v>2</v>
@@ -12351,13 +12351,13 @@
         <v>8.74</v>
       </c>
       <c r="M178" t="n">
-        <v>9.31</v>
+        <v>9.23</v>
       </c>
       <c r="N178" t="n">
         <v>7.6</v>
       </c>
       <c r="O178" t="n">
-        <v>8.536</v>
+        <v>8.52</v>
       </c>
       <c r="P178" t="n">
         <v>1</v>
@@ -12619,13 +12619,13 @@
         <v>9.93</v>
       </c>
       <c r="M182" t="n">
-        <v>6</v>
+        <v>5.99</v>
       </c>
       <c r="N182" t="n">
         <v>2.86</v>
       </c>
       <c r="O182" t="n">
-        <v>7.9665</v>
+        <v>7.9645</v>
       </c>
       <c r="P182" t="n">
         <v>3</v>
@@ -12686,13 +12686,13 @@
         <v>9.33</v>
       </c>
       <c r="M183" t="n">
-        <v>7.56</v>
+        <v>7.52</v>
       </c>
       <c r="N183" t="n">
         <v>5.01</v>
       </c>
       <c r="O183" t="n">
-        <v>8.157</v>
+        <v>8.148999999999999</v>
       </c>
       <c r="P183" t="n">
         <v>2</v>
@@ -12753,13 +12753,13 @@
         <v>8.15</v>
       </c>
       <c r="M184" t="n">
-        <v>9.94</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="N184" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O184" t="n">
-        <v>8.265000000000001</v>
+        <v>8.271000000000001</v>
       </c>
       <c r="P184" t="n">
         <v>1</v>
@@ -12887,13 +12887,13 @@
         <v>9.26</v>
       </c>
       <c r="M186" t="n">
-        <v>7.08</v>
+        <v>7.04</v>
       </c>
       <c r="N186" t="n">
         <v>3.48</v>
       </c>
       <c r="O186" t="n">
-        <v>7.867000000000001</v>
+        <v>7.859000000000001</v>
       </c>
       <c r="P186" t="n">
         <v>1</v>
@@ -12954,13 +12954,13 @@
         <v>8.15</v>
       </c>
       <c r="M187" t="n">
-        <v>9.48</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="N187" t="n">
         <v>4.64</v>
       </c>
       <c r="O187" t="n">
-        <v>7.745499999999999</v>
+        <v>7.727499999999999</v>
       </c>
       <c r="P187" t="n">
         <v>3</v>
@@ -13088,13 +13088,13 @@
         <v>9.33</v>
       </c>
       <c r="M189" t="n">
-        <v>6.26</v>
+        <v>6.23</v>
       </c>
       <c r="N189" t="n">
         <v>2.86</v>
       </c>
       <c r="O189" t="n">
-        <v>7.7095</v>
+        <v>7.703500000000001</v>
       </c>
       <c r="P189" t="n">
         <v>1</v>
@@ -13155,13 +13155,13 @@
         <v>8.44</v>
       </c>
       <c r="M190" t="n">
-        <v>8.220000000000001</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="N190" t="n">
         <v>1.51</v>
       </c>
       <c r="O190" t="n">
-        <v>7.305499999999999</v>
+        <v>7.289499999999999</v>
       </c>
       <c r="P190" t="n">
         <v>3</v>
@@ -13490,13 +13490,13 @@
         <v>9.26</v>
       </c>
       <c r="M195" t="n">
-        <v>7.08</v>
+        <v>7.04</v>
       </c>
       <c r="N195" t="n">
         <v>3.48</v>
       </c>
       <c r="O195" t="n">
-        <v>7.867000000000001</v>
+        <v>7.859000000000001</v>
       </c>
       <c r="P195" t="n">
         <v>1</v>
@@ -13557,13 +13557,13 @@
         <v>8.15</v>
       </c>
       <c r="M196" t="n">
-        <v>9.48</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="N196" t="n">
         <v>4.64</v>
       </c>
       <c r="O196" t="n">
-        <v>7.745499999999999</v>
+        <v>7.727499999999999</v>
       </c>
       <c r="P196" t="n">
         <v>3</v>
@@ -13691,13 +13691,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M198" t="n">
-        <v>7.43</v>
+        <v>7.37</v>
       </c>
       <c r="N198" t="n">
         <v>3.48</v>
       </c>
       <c r="O198" t="n">
-        <v>8.2645</v>
+        <v>8.2525</v>
       </c>
       <c r="P198" t="n">
         <v>2</v>
@@ -13758,13 +13758,13 @@
         <v>8.74</v>
       </c>
       <c r="M199" t="n">
-        <v>9.960000000000001</v>
+        <v>9.99</v>
       </c>
       <c r="N199" t="n">
         <v>7.6</v>
       </c>
       <c r="O199" t="n">
-        <v>8.807</v>
+        <v>8.813000000000001</v>
       </c>
       <c r="P199" t="n">
         <v>1</v>
@@ -13892,13 +13892,13 @@
         <v>9.26</v>
       </c>
       <c r="M201" t="n">
-        <v>6.94</v>
+        <v>6.9</v>
       </c>
       <c r="N201" t="n">
         <v>3.48</v>
       </c>
       <c r="O201" t="n">
-        <v>7.794</v>
+        <v>7.786</v>
       </c>
       <c r="P201" t="n">
         <v>1</v>
@@ -13959,13 +13959,13 @@
         <v>8.52</v>
       </c>
       <c r="M202" t="n">
-        <v>8.49</v>
+        <v>8.42</v>
       </c>
       <c r="N202" t="n">
         <v>3.07</v>
       </c>
       <c r="O202" t="n">
-        <v>7.5075</v>
+        <v>7.4935</v>
       </c>
       <c r="P202" t="n">
         <v>3</v>
@@ -14093,13 +14093,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M204" t="n">
-        <v>7.08</v>
+        <v>7.04</v>
       </c>
       <c r="N204" t="n">
         <v>3.48</v>
       </c>
       <c r="O204" t="n">
-        <v>8.125500000000001</v>
+        <v>8.1175</v>
       </c>
       <c r="P204" t="n">
         <v>2</v>
@@ -14160,13 +14160,13 @@
         <v>8.74</v>
       </c>
       <c r="M205" t="n">
-        <v>9.48</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="N205" t="n">
         <v>7.6</v>
       </c>
       <c r="O205" t="n">
-        <v>8.603</v>
+        <v>8.584999999999999</v>
       </c>
       <c r="P205" t="n">
         <v>1</v>
@@ -14294,13 +14294,13 @@
         <v>9.26</v>
       </c>
       <c r="M207" t="n">
-        <v>6.81</v>
+        <v>6.78</v>
       </c>
       <c r="N207" t="n">
         <v>3.48</v>
       </c>
       <c r="O207" t="n">
-        <v>7.723</v>
+        <v>7.717</v>
       </c>
       <c r="P207" t="n">
         <v>2</v>
@@ -14361,13 +14361,13 @@
         <v>8.15</v>
       </c>
       <c r="M208" t="n">
-        <v>8.93</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="N208" t="n">
         <v>4.64</v>
       </c>
       <c r="O208" t="n">
-        <v>7.4915</v>
+        <v>7.4775</v>
       </c>
       <c r="P208" t="n">
         <v>3</v>
@@ -14495,13 +14495,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M210" t="n">
-        <v>7.28</v>
+        <v>7.23</v>
       </c>
       <c r="N210" t="n">
         <v>3.48</v>
       </c>
       <c r="O210" t="n">
-        <v>8.2075</v>
+        <v>8.1975</v>
       </c>
       <c r="P210" t="n">
         <v>2</v>
@@ -14562,13 +14562,13 @@
         <v>9.039999999999999</v>
       </c>
       <c r="M211" t="n">
-        <v>9.08</v>
+        <v>8.99</v>
       </c>
       <c r="N211" t="n">
         <v>6.37</v>
       </c>
       <c r="O211" t="n">
-        <v>8.605499999999999</v>
+        <v>8.5875</v>
       </c>
       <c r="P211" t="n">
         <v>1</v>
@@ -14830,13 +14830,13 @@
         <v>9.93</v>
       </c>
       <c r="M215" t="n">
-        <v>5.98</v>
+        <v>5.96</v>
       </c>
       <c r="N215" t="n">
         <v>2.86</v>
       </c>
       <c r="O215" t="n">
-        <v>7.9505</v>
+        <v>7.9465</v>
       </c>
       <c r="P215" t="n">
         <v>3</v>
@@ -14897,13 +14897,13 @@
         <v>9.33</v>
       </c>
       <c r="M216" t="n">
-        <v>7.5</v>
+        <v>7.45</v>
       </c>
       <c r="N216" t="n">
         <v>5.01</v>
       </c>
       <c r="O216" t="n">
-        <v>8.123999999999999</v>
+        <v>8.113999999999999</v>
       </c>
       <c r="P216" t="n">
         <v>2</v>
@@ -14964,13 +14964,13 @@
         <v>8.15</v>
       </c>
       <c r="M217" t="n">
-        <v>9.99</v>
+        <v>9.94</v>
       </c>
       <c r="N217" t="n">
         <v>8.449999999999999</v>
       </c>
       <c r="O217" t="n">
-        <v>8.241999999999999</v>
+        <v>8.231999999999999</v>
       </c>
       <c r="P217" t="n">
         <v>1</v>
@@ -15098,13 +15098,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M219" t="n">
-        <v>6.88</v>
+        <v>6.85</v>
       </c>
       <c r="N219" t="n">
         <v>3.48</v>
       </c>
       <c r="O219" t="n">
-        <v>8.0345</v>
+        <v>8.028499999999999</v>
       </c>
       <c r="P219" t="n">
         <v>2</v>
@@ -15165,13 +15165,13 @@
         <v>8.74</v>
       </c>
       <c r="M220" t="n">
-        <v>9.07</v>
+        <v>9</v>
       </c>
       <c r="N220" t="n">
         <v>7.6</v>
       </c>
       <c r="O220" t="n">
-        <v>8.436999999999999</v>
+        <v>8.423</v>
       </c>
       <c r="P220" t="n">
         <v>1</v>
@@ -15299,13 +15299,13 @@
         <v>9.26</v>
       </c>
       <c r="M222" t="n">
-        <v>6.81</v>
+        <v>6.78</v>
       </c>
       <c r="N222" t="n">
         <v>3.48</v>
       </c>
       <c r="O222" t="n">
-        <v>7.723</v>
+        <v>7.717</v>
       </c>
       <c r="P222" t="n">
         <v>2</v>
@@ -15366,13 +15366,13 @@
         <v>8.15</v>
       </c>
       <c r="M223" t="n">
-        <v>8.93</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="N223" t="n">
         <v>4.64</v>
       </c>
       <c r="O223" t="n">
-        <v>7.4915</v>
+        <v>7.4775</v>
       </c>
       <c r="P223" t="n">
         <v>3</v>
@@ -15701,13 +15701,13 @@
         <v>9.26</v>
       </c>
       <c r="M228" t="n">
-        <v>7.04</v>
+        <v>7</v>
       </c>
       <c r="N228" t="n">
         <v>3.48</v>
       </c>
       <c r="O228" t="n">
-        <v>7.847</v>
+        <v>7.839</v>
       </c>
       <c r="P228" t="n">
         <v>1</v>
@@ -15768,13 +15768,13 @@
         <v>8.15</v>
       </c>
       <c r="M229" t="n">
-        <v>9.390000000000001</v>
+        <v>9.31</v>
       </c>
       <c r="N229" t="n">
         <v>4.64</v>
       </c>
       <c r="O229" t="n">
-        <v>7.7065</v>
+        <v>7.6905</v>
       </c>
       <c r="P229" t="n">
         <v>3</v>
@@ -15902,13 +15902,13 @@
         <v>9.630000000000001</v>
       </c>
       <c r="M231" t="n">
-        <v>6.72</v>
+        <v>6.7</v>
       </c>
       <c r="N231" t="n">
         <v>3.48</v>
       </c>
       <c r="O231" t="n">
-        <v>7.9485</v>
+        <v>7.9445</v>
       </c>
       <c r="P231" t="n">
         <v>2</v>
@@ -15969,13 +15969,13 @@
         <v>8.74</v>
       </c>
       <c r="M232" t="n">
-        <v>8.74</v>
+        <v>8.69</v>
       </c>
       <c r="N232" t="n">
         <v>7.6</v>
       </c>
       <c r="O232" t="n">
-        <v>8.286999999999999</v>
+        <v>8.276999999999999</v>
       </c>
       <c r="P232" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Phase I: install calculators, apply scenario fixes, refresh GT/RAG, code changes a-d
- Apply 148 staged scenario fixes; rebuild Test + RAG sheets (65 derived cells)
- Install new HVAC/Appliance/Shower calculators and their tests; regenerate ground truth
- Sync RAG score columns; update README reference ranges and audit_scenarios city map
- Merge provenance into docs/CALCULATOR_PROVENANCE.md (!docs/*.md in .gitignore)
- Duquesne D9 resolved from Supplement 108; 13.75 c/kWh unchanged
- Prompt ablation: CoT max_tokens up to 32768, failed scenario = wrong for Top-1/Top-2
- Lock-protect the consecutive-failure breaker in sentinel_utils
- Regenerate fixed-default baseline; archive pre-rerun outputs to archive/2026-09_pre_rerun/
- Test harness reads archived historical outputs; pin sentinel on misspelled appliance

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JVf7wf3sHYXwFDWcVM4QWD
</commit_message>
<xml_diff>
--- a/Ground Truth/ground_truth_shower.xlsx
+++ b/Ground Truth/ground_truth_shower.xlsx
@@ -766,7 +766,7 @@
         <v>0.29</v>
       </c>
       <c r="O5" t="n">
-        <v>0.7794999999999999</v>
+        <v>0.7795</v>
       </c>
       <c r="P5" t="n">
         <v>3</v>
@@ -900,7 +900,7 @@
         <v>0.85</v>
       </c>
       <c r="O7" t="n">
-        <v>0.8109999999999999</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="P7" t="n">
         <v>2</v>
@@ -1101,7 +1101,7 @@
         <v>0.93</v>
       </c>
       <c r="O10" t="n">
-        <v>0.7509999999999999</v>
+        <v>0.751</v>
       </c>
       <c r="P10" t="n">
         <v>3</v>
@@ -1570,7 +1570,7 @@
         <v>0.5</v>
       </c>
       <c r="O17" t="n">
-        <v>0.6994999999999999</v>
+        <v>0.6995</v>
       </c>
       <c r="P17" t="n">
         <v>1</v>
@@ -1838,7 +1838,7 @@
         <v>0.64</v>
       </c>
       <c r="O21" t="n">
-        <v>0.8119999999999999</v>
+        <v>0.8120000000000001</v>
       </c>
       <c r="P21" t="n">
         <v>1</v>
@@ -1905,7 +1905,7 @@
         <v>0.85</v>
       </c>
       <c r="O22" t="n">
-        <v>0.7999999999999998</v>
+        <v>0.8</v>
       </c>
       <c r="P22" t="n">
         <v>2</v>
@@ -1972,7 +1972,7 @@
         <v>0.22</v>
       </c>
       <c r="O23" t="n">
-        <v>0.7849999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="P23" t="n">
         <v>2</v>
@@ -2039,7 +2039,7 @@
         <v>0.5</v>
       </c>
       <c r="O24" t="n">
-        <v>0.8059999999999999</v>
+        <v>0.806</v>
       </c>
       <c r="P24" t="n">
         <v>1</v>
@@ -2240,7 +2240,7 @@
         <v>0.46</v>
       </c>
       <c r="O27" t="n">
-        <v>0.7129999999999999</v>
+        <v>0.713</v>
       </c>
       <c r="P27" t="n">
         <v>2</v>
@@ -2776,7 +2776,7 @@
         <v>0.5</v>
       </c>
       <c r="O35" t="n">
-        <v>0.6994999999999999</v>
+        <v>0.6995</v>
       </c>
       <c r="P35" t="n">
         <v>1</v>
@@ -3044,7 +3044,7 @@
         <v>0.52</v>
       </c>
       <c r="O39" t="n">
-        <v>0.6839999999999999</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="P39" t="n">
         <v>2</v>
@@ -3446,7 +3446,7 @@
         <v>0.67</v>
       </c>
       <c r="O45" t="n">
-        <v>0.3995000000000001</v>
+        <v>0.3995</v>
       </c>
       <c r="P45" t="n">
         <v>2</v>
@@ -3848,7 +3848,7 @@
         <v>0.76</v>
       </c>
       <c r="O51" t="n">
-        <v>0.8190000000000001</v>
+        <v>0.819</v>
       </c>
       <c r="P51" t="n">
         <v>1</v>
@@ -3915,7 +3915,7 @@
         <v>0.67</v>
       </c>
       <c r="O52" t="n">
-        <v>0.6715000000000001</v>
+        <v>0.6715</v>
       </c>
       <c r="P52" t="n">
         <v>3</v>
@@ -4183,7 +4183,7 @@
         <v>0.15</v>
       </c>
       <c r="O56" t="n">
-        <v>0.6724999999999999</v>
+        <v>0.6725</v>
       </c>
       <c r="P56" t="n">
         <v>3</v>
@@ -4317,7 +4317,7 @@
         <v>0.15</v>
       </c>
       <c r="O58" t="n">
-        <v>0.6854999999999999</v>
+        <v>0.6855</v>
       </c>
       <c r="P58" t="n">
         <v>2</v>
@@ -4585,7 +4585,7 @@
         <v>0.46</v>
       </c>
       <c r="O62" t="n">
-        <v>0.5549999999999999</v>
+        <v>0.555</v>
       </c>
       <c r="P62" t="n">
         <v>1</v>
@@ -4853,7 +4853,7 @@
         <v>0.76</v>
       </c>
       <c r="O66" t="n">
-        <v>0.8190000000000001</v>
+        <v>0.819</v>
       </c>
       <c r="P66" t="n">
         <v>1</v>
@@ -4920,7 +4920,7 @@
         <v>0.93</v>
       </c>
       <c r="O67" t="n">
-        <v>0.7105000000000001</v>
+        <v>0.7105</v>
       </c>
       <c r="P67" t="n">
         <v>3</v>
@@ -5456,7 +5456,7 @@
         <v>0.31</v>
       </c>
       <c r="O75" t="n">
-        <v>0.5005000000000001</v>
+        <v>0.5004999999999999</v>
       </c>
       <c r="P75" t="n">
         <v>2</v>
@@ -5590,7 +5590,7 @@
         <v>0.22</v>
       </c>
       <c r="O77" t="n">
-        <v>0.7849999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="P77" t="n">
         <v>1</v>
@@ -5657,7 +5657,7 @@
         <v>0.46</v>
       </c>
       <c r="O78" t="n">
-        <v>0.7370000000000001</v>
+        <v>0.737</v>
       </c>
       <c r="P78" t="n">
         <v>2</v>
@@ -5791,7 +5791,7 @@
         <v>0.29</v>
       </c>
       <c r="O80" t="n">
-        <v>0.7555000000000001</v>
+        <v>0.7554999999999999</v>
       </c>
       <c r="P80" t="n">
         <v>1</v>
@@ -6193,7 +6193,7 @@
         <v>0.15</v>
       </c>
       <c r="O86" t="n">
-        <v>0.7084999999999999</v>
+        <v>0.7085</v>
       </c>
       <c r="P86" t="n">
         <v>1</v>
@@ -6327,7 +6327,7 @@
         <v>0.57</v>
       </c>
       <c r="O88" t="n">
-        <v>0.3995000000000001</v>
+        <v>0.3995</v>
       </c>
       <c r="P88" t="n">
         <v>3</v>
@@ -6461,7 +6461,7 @@
         <v>0.57</v>
       </c>
       <c r="O90" t="n">
-        <v>0.7174999999999999</v>
+        <v>0.7175</v>
       </c>
       <c r="P90" t="n">
         <v>2</v>
@@ -6595,7 +6595,7 @@
         <v>0.35</v>
       </c>
       <c r="O92" t="n">
-        <v>0.7294999999999999</v>
+        <v>0.7295</v>
       </c>
       <c r="P92" t="n">
         <v>2</v>
@@ -6796,7 +6796,7 @@
         <v>0.35</v>
       </c>
       <c r="O95" t="n">
-        <v>0.6789999999999999</v>
+        <v>0.679</v>
       </c>
       <c r="P95" t="n">
         <v>1</v>
@@ -6997,7 +6997,7 @@
         <v>0.35</v>
       </c>
       <c r="O98" t="n">
-        <v>0.7394999999999999</v>
+        <v>0.7395</v>
       </c>
       <c r="P98" t="n">
         <v>2</v>
@@ -7466,7 +7466,7 @@
         <v>0.46</v>
       </c>
       <c r="O105" t="n">
-        <v>0.6539999999999999</v>
+        <v>0.654</v>
       </c>
       <c r="P105" t="n">
         <v>2</v>
@@ -7533,7 +7533,7 @@
         <v>0.67</v>
       </c>
       <c r="O106" t="n">
-        <v>0.5125000000000001</v>
+        <v>0.5125</v>
       </c>
       <c r="P106" t="n">
         <v>3</v>
@@ -7801,7 +7801,7 @@
         <v>0.46</v>
       </c>
       <c r="O110" t="n">
-        <v>0.5920000000000001</v>
+        <v>0.592</v>
       </c>
       <c r="P110" t="n">
         <v>1</v>
@@ -8002,7 +8002,7 @@
         <v>0.46</v>
       </c>
       <c r="O113" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="P113" t="n">
         <v>1</v>
@@ -8069,7 +8069,7 @@
         <v>0.57</v>
       </c>
       <c r="O114" t="n">
-        <v>0.6190000000000001</v>
+        <v>0.619</v>
       </c>
       <c r="P114" t="n">
         <v>2</v>
@@ -8136,7 +8136,7 @@
         <v>0.67</v>
       </c>
       <c r="O115" t="n">
-        <v>0.5265000000000001</v>
+        <v>0.5265</v>
       </c>
       <c r="P115" t="n">
         <v>3</v>
@@ -8538,7 +8538,7 @@
         <v>0.67</v>
       </c>
       <c r="O121" t="n">
-        <v>0.5255000000000001</v>
+        <v>0.5255</v>
       </c>
       <c r="P121" t="n">
         <v>3</v>
@@ -8672,7 +8672,7 @@
         <v>0.46</v>
       </c>
       <c r="O123" t="n">
-        <v>0.6260000000000001</v>
+        <v>0.626</v>
       </c>
       <c r="P123" t="n">
         <v>2</v>
@@ -9074,7 +9074,7 @@
         <v>0.46</v>
       </c>
       <c r="O129" t="n">
-        <v>0.6260000000000001</v>
+        <v>0.626</v>
       </c>
       <c r="P129" t="n">
         <v>2</v>
@@ -9275,7 +9275,7 @@
         <v>0.76</v>
       </c>
       <c r="O132" t="n">
-        <v>0.8190000000000001</v>
+        <v>0.819</v>
       </c>
       <c r="P132" t="n">
         <v>1</v>
@@ -9342,7 +9342,7 @@
         <v>0.67</v>
       </c>
       <c r="O133" t="n">
-        <v>0.6715000000000001</v>
+        <v>0.6715</v>
       </c>
       <c r="P133" t="n">
         <v>3</v>
@@ -9476,7 +9476,7 @@
         <v>0.46</v>
       </c>
       <c r="O135" t="n">
-        <v>0.7149999999999999</v>
+        <v>0.715</v>
       </c>
       <c r="P135" t="n">
         <v>2</v>
@@ -9811,7 +9811,7 @@
         <v>0.15</v>
       </c>
       <c r="O140" t="n">
-        <v>0.6034999999999999</v>
+        <v>0.6035</v>
       </c>
       <c r="P140" t="n">
         <v>1</v>
@@ -10012,7 +10012,7 @@
         <v>0.15</v>
       </c>
       <c r="O143" t="n">
-        <v>0.6764999999999999</v>
+        <v>0.6765</v>
       </c>
       <c r="P143" t="n">
         <v>2</v>
@@ -10213,7 +10213,7 @@
         <v>0.64</v>
       </c>
       <c r="O146" t="n">
-        <v>0.7374999999999999</v>
+        <v>0.7375</v>
       </c>
       <c r="P146" t="n">
         <v>1</v>
@@ -10414,7 +10414,7 @@
         <v>0.35</v>
       </c>
       <c r="O149" t="n">
-        <v>0.7294999999999999</v>
+        <v>0.7295</v>
       </c>
       <c r="P149" t="n">
         <v>1</v>
@@ -10749,7 +10749,7 @@
         <v>0.67</v>
       </c>
       <c r="O154" t="n">
-        <v>0.5455000000000001</v>
+        <v>0.5455</v>
       </c>
       <c r="P154" t="n">
         <v>3</v>
@@ -10816,7 +10816,7 @@
         <v>0.15</v>
       </c>
       <c r="O155" t="n">
-        <v>0.6769999999999999</v>
+        <v>0.677</v>
       </c>
       <c r="P155" t="n">
         <v>1</v>
@@ -11151,7 +11151,7 @@
         <v>0.67</v>
       </c>
       <c r="O160" t="n">
-        <v>0.5255000000000001</v>
+        <v>0.5255</v>
       </c>
       <c r="P160" t="n">
         <v>3</v>
@@ -11486,7 +11486,7 @@
         <v>0.46</v>
       </c>
       <c r="O165" t="n">
-        <v>0.7149999999999999</v>
+        <v>0.715</v>
       </c>
       <c r="P165" t="n">
         <v>2</v>
@@ -11620,7 +11620,7 @@
         <v>0.22</v>
       </c>
       <c r="O167" t="n">
-        <v>0.7849999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="P167" t="n">
         <v>2</v>
@@ -11687,7 +11687,7 @@
         <v>0.35</v>
       </c>
       <c r="O168" t="n">
-        <v>0.7825000000000001</v>
+        <v>0.7825</v>
       </c>
       <c r="P168" t="n">
         <v>3</v>
@@ -11955,7 +11955,7 @@
         <v>0.46</v>
       </c>
       <c r="O172" t="n">
-        <v>0.7149999999999999</v>
+        <v>0.715</v>
       </c>
       <c r="P172" t="n">
         <v>3</v>
@@ -12022,7 +12022,7 @@
         <v>0.22</v>
       </c>
       <c r="O173" t="n">
-        <v>0.7649999999999999</v>
+        <v>0.765</v>
       </c>
       <c r="P173" t="n">
         <v>1</v>
@@ -12156,7 +12156,7 @@
         <v>0.46</v>
       </c>
       <c r="O175" t="n">
-        <v>0.7069999999999999</v>
+        <v>0.707</v>
       </c>
       <c r="P175" t="n">
         <v>3</v>
@@ -12223,7 +12223,7 @@
         <v>0.22</v>
       </c>
       <c r="O176" t="n">
-        <v>0.7849999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="P176" t="n">
         <v>1</v>
@@ -12491,7 +12491,7 @@
         <v>0.5</v>
       </c>
       <c r="O180" t="n">
-        <v>0.7699999999999999</v>
+        <v>0.77</v>
       </c>
       <c r="P180" t="n">
         <v>2</v>
@@ -12558,7 +12558,7 @@
         <v>0.85</v>
       </c>
       <c r="O181" t="n">
-        <v>0.7749999999999999</v>
+        <v>0.775</v>
       </c>
       <c r="P181" t="n">
         <v>1</v>
@@ -12692,7 +12692,7 @@
         <v>0.5</v>
       </c>
       <c r="O183" t="n">
-        <v>0.7324999999999999</v>
+        <v>0.7325</v>
       </c>
       <c r="P183" t="n">
         <v>2</v>
@@ -12759,7 +12759,7 @@
         <v>0.85</v>
       </c>
       <c r="O184" t="n">
-        <v>0.7064999999999999</v>
+        <v>0.7065</v>
       </c>
       <c r="P184" t="n">
         <v>3</v>
@@ -13161,7 +13161,7 @@
         <v>0.15</v>
       </c>
       <c r="O190" t="n">
-        <v>0.6539999999999999</v>
+        <v>0.654</v>
       </c>
       <c r="P190" t="n">
         <v>3</v>
@@ -13228,7 +13228,7 @@
         <v>0.22</v>
       </c>
       <c r="O191" t="n">
-        <v>0.7729999999999999</v>
+        <v>0.773</v>
       </c>
       <c r="P191" t="n">
         <v>1</v>
@@ -13965,7 +13965,7 @@
         <v>0.31</v>
       </c>
       <c r="O202" t="n">
-        <v>0.6729999999999999</v>
+        <v>0.673</v>
       </c>
       <c r="P202" t="n">
         <v>3</v>
@@ -14233,7 +14233,7 @@
         <v>0.22</v>
       </c>
       <c r="O206" t="n">
-        <v>0.7529999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="P206" t="n">
         <v>1</v>
@@ -14367,7 +14367,7 @@
         <v>0.46</v>
       </c>
       <c r="O208" t="n">
-        <v>0.6539999999999999</v>
+        <v>0.654</v>
       </c>
       <c r="P208" t="n">
         <v>3</v>
@@ -14434,7 +14434,7 @@
         <v>0.22</v>
       </c>
       <c r="O209" t="n">
-        <v>0.7849999999999999</v>
+        <v>0.785</v>
       </c>
       <c r="P209" t="n">
         <v>3</v>
@@ -14501,7 +14501,7 @@
         <v>0.35</v>
       </c>
       <c r="O210" t="n">
-        <v>0.7905000000000001</v>
+        <v>0.7905</v>
       </c>
       <c r="P210" t="n">
         <v>2</v>
@@ -14635,7 +14635,7 @@
         <v>0.29</v>
       </c>
       <c r="O212" t="n">
-        <v>0.7625000000000001</v>
+        <v>0.7625</v>
       </c>
       <c r="P212" t="n">
         <v>3</v>
@@ -14836,7 +14836,7 @@
         <v>0.29</v>
       </c>
       <c r="O215" t="n">
-        <v>0.7300000000000001</v>
+        <v>0.73</v>
       </c>
       <c r="P215" t="n">
         <v>1</v>
@@ -14903,7 +14903,7 @@
         <v>0.5</v>
       </c>
       <c r="O216" t="n">
-        <v>0.7294999999999999</v>
+        <v>0.7295</v>
       </c>
       <c r="P216" t="n">
         <v>2</v>
@@ -15037,7 +15037,7 @@
         <v>0.22</v>
       </c>
       <c r="O218" t="n">
-        <v>0.7380000000000001</v>
+        <v>0.738</v>
       </c>
       <c r="P218" t="n">
         <v>2</v>
@@ -15104,7 +15104,7 @@
         <v>0.35</v>
       </c>
       <c r="O219" t="n">
-        <v>0.7294999999999999</v>
+        <v>0.7295</v>
       </c>
       <c r="P219" t="n">
         <v>3</v>
@@ -15238,7 +15238,7 @@
         <v>0.22</v>
       </c>
       <c r="O221" t="n">
-        <v>0.7529999999999999</v>
+        <v>0.753</v>
       </c>
       <c r="P221" t="n">
         <v>1</v>
@@ -15372,7 +15372,7 @@
         <v>0.46</v>
       </c>
       <c r="O223" t="n">
-        <v>0.6539999999999999</v>
+        <v>0.654</v>
       </c>
       <c r="P223" t="n">
         <v>3</v>
@@ -15439,7 +15439,7 @@
         <v>0.22</v>
       </c>
       <c r="O224" t="n">
-        <v>0.7729999999999999</v>
+        <v>0.773</v>
       </c>
       <c r="P224" t="n">
         <v>1</v>
@@ -15640,7 +15640,7 @@
         <v>0.22</v>
       </c>
       <c r="O227" t="n">
-        <v>0.7589999999999999</v>
+        <v>0.759</v>
       </c>
       <c r="P227" t="n">
         <v>1</v>
@@ -15774,7 +15774,7 @@
         <v>0.46</v>
       </c>
       <c r="O229" t="n">
-        <v>0.6799999999999999</v>
+        <v>0.68</v>
       </c>
       <c r="P229" t="n">
         <v>3</v>
@@ -16042,7 +16042,7 @@
         <v>0.15</v>
       </c>
       <c r="O233" t="n">
-        <v>0.6329999999999999</v>
+        <v>0.633</v>
       </c>
       <c r="P233" t="n">
         <v>1</v>
@@ -16243,7 +16243,7 @@
         <v>0.29</v>
       </c>
       <c r="O236" t="n">
-        <v>0.7794999999999999</v>
+        <v>0.7795</v>
       </c>
       <c r="P236" t="n">
         <v>3</v>
@@ -16377,7 +16377,7 @@
         <v>0.85</v>
       </c>
       <c r="O238" t="n">
-        <v>0.8109999999999999</v>
+        <v>0.8110000000000001</v>
       </c>
       <c r="P238" t="n">
         <v>2</v>
@@ -16444,7 +16444,7 @@
         <v>0.15</v>
       </c>
       <c r="O239" t="n">
-        <v>0.6839999999999999</v>
+        <v>0.6840000000000001</v>
       </c>
       <c r="P239" t="n">
         <v>1</v>
@@ -16511,7 +16511,7 @@
         <v>0.46</v>
       </c>
       <c r="O240" t="n">
-        <v>0.6379999999999999</v>
+        <v>0.638</v>
       </c>
       <c r="P240" t="n">
         <v>2</v>
@@ -16578,7 +16578,7 @@
         <v>0.67</v>
       </c>
       <c r="O241" t="n">
-        <v>0.4985000000000001</v>
+        <v>0.4985</v>
       </c>
       <c r="P241" t="n">
         <v>3</v>

</xml_diff>